<commit_message>
Add evaluation pipeline cleanup and export tooling
</commit_message>
<xml_diff>
--- a/data_awal.xlsx
+++ b/data_awal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SKRIPSI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uph365-my.sharepoint.com/personal/01085220003_student_uph_edu/Documents/SKRIPSI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67FC2845-8B74-4E2F-9412-4D7CD715F6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{28CFE712-C0B3-40BC-B89E-5603FDB7012E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9DD10947-EA4E-42EA-8B01-D1CA78034524}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
   <si>
     <t>Pertanyaan</t>
   </si>
@@ -59,41 +59,6 @@
   <si>
     <t>Berdasarkan artikel Designing secure blockchain-based authentication and key management
 mechanism for Internet of Drones applications, jelaskan mengenai Blockchain implementation phase</t>
-  </si>
-  <si>
-    <t>Jelaskan mengenai Comparisons of communicational overhead pada artikel ilmiah A blockchain and IPFS-Aided anonymous traitor tracing scheme
-based on puncturable encryption in Industrial Internet of Things</t>
-  </si>
-  <si>
-    <t>Berikan abstrak dari A cloud-assisted anonymous and privacy-preserving authentication scheme
-for internet of medical things</t>
-  </si>
-  <si>
-    <t>Apa saja Research limitations pada artikel ilmiah A comprehensive review of cybersecurity vulnerabilities, threats, and
-solutions for the Internet of Things at the network-cum-application layer</t>
-  </si>
-  <si>
-    <t>Apa motivation yang dibahas pada dokumen ilmiah A hybrid PKI and spiking neural network approach for enhancing security
-and energy efficiency in IoMT-based healthcare 5.0?</t>
-  </si>
-  <si>
-    <t>Siapa saja penulis jurnal ilmiah A machine learning approach for detecting cybersecurity vulnerabilities in
-the internet of medical things?</t>
-  </si>
-  <si>
-    <t>Apa framework yang diusulkan pada dokumen ilmiah A new design of arithmetic and logic unit for enhancing the security of
-future internet of things devices using quantum-dot technology?</t>
-  </si>
-  <si>
-    <t>Apa konklusi dari dokumen ilmiah Blockchain based lightweight authentication scheme for internet of things
-using lattice encryption algorithm</t>
-  </si>
-  <si>
-    <t>Apa saja highlight dari dokumen ilmiah Distributed Ledgers and Security Mechanisms on Radio Access Networks: A Systematic Review</t>
-  </si>
-  <si>
-    <t>jelaskan mengenai Cross-domain data sharing scheme pada dokumen ilmiah Efficient and secure cross-domain data sharing scheme with traceability for
-Industrial Internet?</t>
   </si>
   <si>
     <t>During this step, we present the specifics of the blockchain. It is a
@@ -238,7 +203,33 @@
 technologies, opportunities and challenges</t>
   </si>
   <si>
+    <t>As an integrant of SCs, SHs and SBs equipped with advanced communication technologies and IoT can provide a variety of
+services to their inhabitants through adaptations and responsiveness. However, the conventional communication systems deteriorate
+to provide satisfactory performance due to the high data generated by the IoT devices. The 6G-IoT system will lead to intelligent and
+autonomous connected systems that can pave the way to turn the concept of SCs from hype to reality. In this paper, we surveyed the
+existing literature on SHs and SBs and we investigated the enabling 6G technologies in the context of SHs and SBs with an emphasis
+on IoT enabled SHs and SBs, its major requirements, advanced ICT, and enabling 6G technologies followed by the key challenges and
+opportunities. Given the significance of 6G and IoT in SCs, this survey article provide a guideline and helpful resources in defining
+the future research direction in modeling of future SHs and SBs. Keeping in view the challenges, the advanced ML techniques
+needs to be explored for integrated communication and sensing in SHs and SBs such as transformer and diffusion models. On the
+other hand, cloud–edge collaboration technologies such as federated learning, edge intelligence and distributed optimization can be
+considered to enhance intelligence in SHs and SBs. Similarly, the performance evaluation and optimization of the multiple coexisted
+technologies such as JCAS, VLC and sensing, BC, and RIS aided smart indoor environment needs further exploration in future. More
+specifically, advances in RIS architectures such as simultaneous transmission and reflection (STAR)-RIS and optical RIS (ORIS) for
+the SH and SB applications is one of the trending topic that needs to be explored. Moreover, explainable AI along with the digital
+twin needs to be considered for SHs and SBs applications. On the other hand, the interoperability of multiple technologies in case
+of interconnected homes and building along with the healthcare systems is challenging and needs special consideration</t>
+  </si>
+  <si>
+    <t>Jelaskan mengenai Comparisons of communicational overhead pada artikel ilmiah A blockchain and IPFS-Aided anonymous traitor tracing scheme
+based on puncturable encryption in Industrial Internet of Things</t>
+  </si>
+  <si>
     <t>As an integrant of SCs, SHs and SBs equipped with advanced communication technologies and IoT can provide a variety of services to their inhabitants through adaptations and responsiveness. However, the conventional communication systems deteriorate to provide satisfactory performance due to the high data generated by the IoT devices. The 6G-IoT system will lead to intelligent and autonomous connected systems that can pave the way to turn the concept of SCs from hype to reality. In this paper, we surveyed the existing literature on SHs and SBs and we investigated the enabling 6G technologies in the context of SHs and SBs with an emphasis on IoT enabled SHs and SBs, its major requirements, advanced ICT, and enabling 6G technologies followed by the key challenges and opportunities. Given the significance of 6G and IoT in SCs, this survey article provide a guideline and helpful resources in defining the future research direction in modeling of future SHs and SBs. Keeping in view the challenges, the advanced ML techniques needs to be explored for integrated communication and sensing in SHs and SBs such as transformer and diffusion models. On the other hand, cloud–edge collaboration technologies such as federated learning, edge intelligence and distributed optimization can be considered to enhance intelligence in SHs and SBs. Similarly, the performance evaluation and optimization of the multiple coexisted technologies such as JCAS, VLC and sensing, BC, and RIS aided smart indoor environment needs further exploration in future. More specifically, advances in RIS architectures such as simultaneous transmission and reflection (STAR)-RIS and optical RIS (ORIS) for the SH and SB applications is one of the trending topic that needs to be explored. Moreover, explainable AI along with the digital twin needs to be considered for SHs and SBs applications. On the other hand, the interoperability of multiple technologies in case of interconnected homes and building along with the healthcare systems is challenging and needs special consideration.</t>
+  </si>
+  <si>
+    <t>Berikan abstrak dari A cloud-assisted anonymous and privacy-preserving authentication scheme
+for internet of medical things</t>
   </si>
   <si>
     <t>With the rapid advancement of the Internet of Medical Things (IoMT) and the increasing adoption of cloud
@@ -258,12 +249,23 @@
 solutions.</t>
   </si>
   <si>
+    <t>Apa saja Research limitations pada artikel ilmiah A comprehensive review of cybersecurity vulnerabilities, threats, and
+solutions for the Internet of Things at the network-cum-application layer</t>
+  </si>
+  <si>
     <t>The article, while comprehensive, does not encompass all contem
 porary IoT research, concentrating instead on studies conducted
 tween 2009 and 2024. This limitation may affect its pertinence to nascent trends and technologies that have not yet undergone substantial examination. The study may possess diminished empirical significance due to its reliance on secondary data and literature reviews, as it lacks direct evidence to substantiate its assertions and does not conduct original experimental validation.
 Although the article effectively classifies IoT applications, general
 ization poses challenges due to IoT domains’ diversity and rapid expansion. Specific sectors, like healthcare and industrial IoT, present distinct challenges that necessitate specialized research and solutions. Moreover, although the study’s recommendations are plausible and attainable, substantial obstacles may exist. Scalability, financial
 tions, and compatibility with many IoT platforms may all hinder the practical feasibility of suggested security solutions. These constraints highlight the need for additional enhancement and contextualization to guarantee that the study’s conclusions and recommendations can be effectively used across diverse IoT scenarios.</t>
+  </si>
+  <si>
+    <t>Jelaskan Certificate-less public key encryption pada dokumen ilmiah Edge-assisted lightweight message authentication for Industrial Internet of
+Things</t>
+  </si>
+  <si>
+    <t>Certificate-less public key encryption (CL-PKC) is a model that utilizes public key encryption while avoiding the inherent key escrow associated with identity-based encryption, and it does not require certificates to verify the authenticity of public keys. In the CL-PKC system, Key Generation Center (KGC) provides entities with partial private keys, which the entities then combine with secret information to generate their actual private keys. Additionally, entities compute their public keys by combining their secret information with the KGC’s public parameters. In this framework, the KGC is unable to access the entities’ private keys, thus mitigating the key escrow issue. More details can be found in [50].</t>
   </si>
   <si>
     <t>Apa itu Data sharing based on blockchain pada artikel ilmiah A data sharing scheme based on blockchain for privacy protection
@@ -414,9 +416,6 @@
 system in Industrial Internet of Things?</t>
   </si>
   <si>
-    <t>In the healthcare 5.0 era, IoMT is revolutionizing patient care by achieving seamless connectivity and real-time access to data. Still, significant issues remain in terms of secure energy-efficient data transmission. Protecting health information from unauthorized access to patient data and efficient utilization of energy in resource-constrained settings is very important. The requirements and actual motivation for this work relate to the meeting of the above two challenges jointly through the design of an effective framework that will rely on PKI for secure communication, spike neural networks for precise anomaly detection, and ZOA for energy optimization. Such a comprehensive approach will make privacy stronger, network life longer, and healthcare IoMT systems operate in a reliable and effective way.</t>
-  </si>
-  <si>
     <t>The proposed hybrid IDS utilises machine learning and optimisation techniques to enhance the security of industrial IoT networks using blockchain technology. Incorporating blockchain technology ensures that data is immutable, that trust is created, and that communications among IoT devices are secure. In addition to improving threat detection accuracy, XGBoost minimises false positives in AFSO Optimization. This model outperforms existing models in high detection accuracy (97.43%) using the BOT-IoT dataset. Using blockchains for intrusion detection and security of IIoT environments has been found to be effective in reducing cyber threats and improving security. Developing real-time deployment scenarios and adaptive learning models will enhance IDS resilience when dealing with evolving cyber threats in the future. Future work will analyze the long-term viability of the block
 chain ledger in handling high-frequency security events, focusing</t>
   </si>
@@ -460,7 +459,57 @@
 cause, and assess the harm of an incident by using audit trails.</t>
   </si>
   <si>
+    <t>Apa motivation yang dibahas pada dokumen ilmiah A hybrid PKI and spiking neural network approach for enhancing security
+and energy efficiency in IoMT-based healthcare 5.0?</t>
+  </si>
+  <si>
+    <t>In the healthcare 5.0 era, IoMT is revolutionizing patient care by achieving seamless connectivity and real-time access to data. Still, significant issues remain in terms of secure energy-efficient data transmission. Protecting health information from unauthorized access to patient data and efficient utilization of energy in resource-constrained settings is very important. The requirements and actual motivation for this work relate to the meeting of the above two challenges jointly through the design of an effective framework that will rely on PKI for secure communication, spike neural networks for precise anomaly detection, and ZOA for energy optimization. Such a comprehensive approach will make privacy stronger, network life longer, and healthcare IoMT systems operate in a reliable and effective way.</t>
+  </si>
+  <si>
+    <t>Jelaskan Neural networks data pada dokumen ilmiah Towards an intelligent and automatic irrigation system based on internet of
+things with authentication feature in VANET</t>
+  </si>
+  <si>
+    <t>Advancements in sensor technology and the widespread adoption of
+smart solutions across various domains, including environmental, industrial,
+and medical sectors, have created numerous opportunities for
+innovative applications [22,23]. Applications simultaneously are
+becoming more complex; thus, the end-user needs a platform that carries
+these applications to support mobility and flexibility to act more adaptively
+to new requirements. Also, when designing the system, it must be
+taken wider than what was before. Typically, applications based on
+WSNs, broadcast, monitoring systems, IoT, and peer-to-peer relay we
+can rely on including cloud services. Time and location are the most
+stringent restrictions for these systems and services. Thus, the situation
+is more stringent in terms of multimedia data transmission, and to
+overcome network problems special processing and protocols are used
+for multimedia applications (broadcast, telephone, etc.) [24,25].
+Because of the flow of data packets in the network, the Quality of Services
+(QoS) must be considered, such as delay, data loss rate, and costs,
+to maintain the quality of data transmission. Therefore, routing is a
+crucial factor that has a significant impact on packet switching in
+network performance.
+Since of the constraints governing the process of exchanging packets
+on the network, routing algorithms should provide the most appropriate
+path (optimum) for the network according to the traffic volume and QoS
+conditions. Therefore, arithmetic operations must be performed when
+the transmission command is received between the network’s routers.
+Neural networks are at the forefront of these operations because they
+perform enormous operations to manage the situation in conjunction
+with the rest of the transmission process procedures. This study investigates
+using the neural network, which is fully compatible with the
+multi-routing of Internet networks.</t>
+  </si>
+  <si>
+    <t>Siapa saja penulis jurnal ilmiah A machine learning approach for detecting cybersecurity vulnerabilities in
+the internet of medical things?</t>
+  </si>
+  <si>
     <t>Ukamaka Oragwu, Benjamin Aziz ∗, Shahadate Rezvy</t>
+  </si>
+  <si>
+    <t>Apa framework yang diusulkan pada dokumen ilmiah A new design of arithmetic and logic unit for enhancing the security of
+future internet of things devices using quantum-dot technology?</t>
   </si>
   <si>
     <t>Modern smart environments rely on IoT devices since they have the potential to ensure a high level of convenience and real-time data transfer between various systems (Elgazzar et al., 2022). These are sensors, actuators, and other devices that collect huge volumes of data and enable many applications in smart cities (Elgazzar et al., 2022). Thus, there are growing demands to ensure the security of these IoT devices and computational elements. Moreover, Fig. 3also shows how the ALU is critical in this integrated IoT ecosystem. The ALU processes data collected from IoT sensors and devices and enables local compu
@@ -603,6 +652,10 @@
 (4) Performance tests and security analysis indicate that our scheme offers better security while enhancing performance comparedto alternative algorithms. We achieve shorter identity authentication times, making it more suitable for practical applications in theIIoT.</t>
   </si>
   <si>
+    <t>Apa konklusi dari dokumen ilmiah Blockchain based lightweight authentication scheme for internet of things
+using lattice encryption algorithm</t>
+  </si>
+  <si>
     <t>This paper proposed a novel and lightweight authentication scheme
 for securing interconnected devices in the rapidly growing Internet
 of Things (IoT) environment. Recognizing the limitations of traditional
@@ -628,11 +681,18 @@
 and performance.</t>
   </si>
   <si>
+    <t>Apa saja highlight dari dokumen ilmiah Distributed Ledgers and Security Mechanisms on Radio Access Networks: A Systematic Review</t>
+  </si>
+  <si>
     <t>The evolution of mobile communication based on openness, softwarization, and virtualization inserts new vulnerabilities into networks.
 • The increasing number of connected devices, especially IoT ones, is a security attention point in mobile networks.
 • Various security mechanisms, including Distributed ledger technologies (DLT), may enhance RAN security once these technologies can increase system
 resilience.
 • Other security approaches may also address RAN security issues.</t>
+  </si>
+  <si>
+    <t>jelaskan mengenai Cross-domain data sharing scheme pada dokumen ilmiah Efficient and secure cross-domain data sharing scheme with traceability for
+Industrial Internet?</t>
   </si>
   <si>
     <t>The above schemes are suitable for single-domain environments andlack the capability to support multi-domain data sharing, which is notconducive to realizing the full value of data and limits opportunitiesfor innovation and collaboration. To solve the problem, Shen et al.proposed a framework to enhance the security of device authenticationin the cross-domain Industrial Internet of Things (IIoT) environmentby using blockchain technology [21]. Chi et al. proposed an effectiveand secure cross-domain data sharing protocol for the IIoT, which usesidentity authentication technology to achieve access control of data andblockchain technology to ensure data security and traceability [10].The scheme proposed in Ref. [22] provides a cross-domain data sharingscheme based on centralized cloud platforms and blockchain that main-tains trust relationships between different domains for manufacturingcollaboration. Cheng et al. combined edge computing and blockchaintechnologies with public key encryption with keyword search (PEKS)to achieve efficient and secure cross-domain data sharing, while en-suring privacy protection and data integrity [23]. Yu et al. proposea blockchain-based enhanced security access control scheme that ad-dresses the semi-trustworthiness of smart factories cloud platformsin IIoT while protecting data security [24]. Zeng et al. presenteda blockchain-based inter-domain data sharing protocol using zero-knowledge proof and key agreement protocol to guarantee data securityand privacy in IIoT. However, data encryption adopts symmetric en-cryption (SE), which can only perform one-to-one access control, andthe access policy is not flexible enough [25]. Despite the prospects arepromising, the combination of blockchain and data governance stillfaces some challenges, and the privacy of the data still need to beexplored [26].
@@ -739,6 +799,9 @@
     <t>Blockchain technology is used in SG systems to improve the security, transparency, and efficiency of energy management. Its performance is evaluated using three key cost metrics: computation cost, communication cost, and smart-contract execution cost. Computation cost measures the resources required for energy transactions, while communication cost assesses data exchange among grid nodes. Smart-contract execution cost is critical, encompassing both one-time deployment costs and ongoing costs for regular interactions.</t>
   </si>
   <si>
+    <t>Apa konklusi  dari artikel ilmiah Toward zero trust in 5G Industrial Internet collaboration system?</t>
+  </si>
+  <si>
     <t>In this paper, we introduced the security issues in the 5G Industrial
 Internet collaboration system, and presented an overview of the
 current ZTA. Then, we presented a gap analysis between existing techniques
@@ -768,56 +831,97 @@
 multiple and increasingly sophisticated attacks.</t>
   </si>
   <si>
-    <t>Apa konklusi  dari artikel ilmiah Toward zero trust in 5G Industrial Internet collaboration system?</t>
-  </si>
-  <si>
-    <t>Advancements in sensor technology and the widespread adoption of
-smart solutions across various domains, including environmental, industrial,
-and medical sectors, have created numerous opportunities for
-innovative applications [22,23]. Applications simultaneously are
-becoming more complex; thus, the end-user needs a platform that carries
-these applications to support mobility and flexibility to act more adaptively
-to new requirements. Also, when designing the system, it must be
-taken wider than what was before. Typically, applications based on
-WSNs, broadcast, monitoring systems, IoT, and peer-to-peer relay we
-can rely on including cloud services. Time and location are the most
-stringent restrictions for these systems and services. Thus, the situation
-is more stringent in terms of multimedia data transmission, and to
-overcome network problems special processing and protocols are used
-for multimedia applications (broadcast, telephone, etc.) [24,25].
-Because of the flow of data packets in the network, the Quality of Services
-(QoS) must be considered, such as delay, data loss rate, and costs,
-to maintain the quality of data transmission. Therefore, routing is a
-crucial factor that has a significant impact on packet switching in
-network performance.
-Since of the constraints governing the process of exchanging packets
-on the network, routing algorithms should provide the most appropriate
-path (optimum) for the network according to the traffic volume and QoS
-conditions. Therefore, arithmetic operations must be performed when
-the transmission command is received between the network’s routers.
-Neural networks are at the forefront of these operations because they
-perform enormous operations to manage the situation in conjunction
-with the rest of the transmission process procedures. This study investigates
-using the neural network, which is fully compatible with the
-multi-routing of Internet networks.</t>
-  </si>
-  <si>
-    <t>Jelaskan Neural networks data pada dokumen ilmiah Towards an intelligent and automatic irrigation system based on internet of
-things with authentication feature in VANET</t>
-  </si>
-  <si>
-    <t>Jelaskan Certificate-less public key encryption pada dokumen ilmiah Edge-assisted lightweight message authentication for Industrial Internet of
-Things</t>
-  </si>
-  <si>
-    <t>Certificate-less public key encryption (CL-PKC) is a model that utilizes public key encryption while avoiding the inherent key escrow associated with identity-based encryption, and it does not require certificates to verify the authenticity of public keys. In the CL-PKC system, Key Generation Center (KGC) provides entities with partial private keys, which the entities then combine with secret information to generate their actual private keys. Additionally, entities compute their public keys by combining their secret information with the KGC’s public parameters. In this framework, the KGC is unable to access the entities’ private keys, thus mitigating the key escrow issue. More details can be found in [50].</t>
+    <t>Apa itu Application layer yang dijelaskan pada artikel ilmiah Privacy and security of wearable internet of things: A scoping review and
+conceptual framework development for safety and health management
+in construction</t>
+  </si>
+  <si>
+    <t>The application layer is the end-user of the cycle where the infor_x0002_mation obtained and processed is used for the intended purpose. This
+layer promotes the development of an IoT system as it is the reason for
+the development of the entire system (Farooq et al., 2015). In the con_x0002_struction industry, real-time information on construction workers and
+the work environment could help safety officers and construction
+workers make more informed proactive decisions to improve safety and
+health performance. For instance, WIoT can monitor the vital signs and
+locations of construction workers in real-time. This information can be
+instantly relayed to safety officers, who can respond swiftly in the event
+of an emergency or if a worker’s health is compromised. Such proactive
+measures can save lives and prevent accidents. In some cases, this in_x0002_formation contains personal information that can be used to identify
+individuals, thereby presenting the need to provide security measures to
+protect such information.</t>
+  </si>
+  <si>
+    <t>Jelaskan discussion pada paper ilmiah Security and privacy in edge computing: a survey of electric vehicles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In this paper, we present a holistic overview of EC and highlight its
+key characteristics such as location awareness, its distributed nature,
+and support from large-scale IoT applications. We have discussed the
+security risks and challenges associated with the core infrastructure, ac_x0002_cess networks, and data security and privacy in EC.
+Looking ahead, EC faces several challenges. First, ensuring robust
+security of the core infrastructure and access networks will be crucial
+for protecting against potential cyberattacks and data breaches. Second,
+as EC continues to grow in scale, it will be necessary to develop stan_x0002_dardized security protocols and mechanisms that can be applied univer_x0002_sally. Third, as the amount of sensitive data at edge servers increases,
+the development of more effective privacy preservation techniques is
+becoming essential for safeguarding users’ information. Additionally,
+the tradeoff between security and performance metrics is expected to be
+another critical challenge in EC.
+Moreover, methods for quantifying and measuring privacy risks and
+benefits in EC remain an ongoing area of study. Standardizing pri_x0002_vacy quantification methodologies will be vital for evaluating the effec_x0002_tiveness of privacy protection methods and ensuring compliance with
+regulations. Finally, EC involves collaboration among multiple stake_x0002_holders, including device manufacturers, network operators, and service
+providers. Coordinating security efforts among these diverse entities
+and establishing effective governance mechanisms will be essential for
+developing holistic and collaborative solutions for EC security.
+Our study clarifies the importance of security and privacy in EC and
+presents a review of existing approaches developed in the domains of
+offloading, the IoV, and smart grids. The challenges identified in this
+paper point to a need for continuous efforts in developing secure and
+privacy-preserving solutions in the future.
+</t>
+  </si>
+  <si>
+    <t>Apa itu Abused domain categorization pada artikel ilmiah Web of shadows: Investigating malware abuse of internet services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In addition to the discussion in Section 3, we analyze what kind of
+services are being abused adding context to RQ3. To classify domains,
+we leverage the information available in the 22K VT reports. VT runs
+user-submitted domains through various commercial providers that cat_x0002_egorize the domains into classes that roughly capture industrial sectors
+(e.g., Information Technology, Education, Games). We observe 11 such
+providers used by VT. For each provider, Fig. 6 shows the fraction
+of domains for which the provider outputs at least one category. The
+provider with the highest coverage is Forcepoint, which classifies 82%
+of the 22K domains, followed by Xcitum (72%), and BitDefender (68%).
+A provider may output multiple categories for the same domain. To
+obtain a category for each domain, we favor the coverage criteria.
+For each domain, we first assign the category from the provider with
+the largest coverage (i.e., Forcepoint). If that provider does not return
+a category for the domain, we move to the next provider in terms
+of coverage, and so on until a category is found. Since categories
+used by each provider may not map one-to-one, we manually build a
+mapping to solve disagreements. Using this methodology, we are able
+to categorize 95% of the 22K domains into 63 categories. For each of
+these categories, Fig. 7 shows the probability density function of being
+ranked in the specific range of the Tranco 1M list. Each domain is
+weighted by the number of reports it receives. The most popular cate_x0002_gory is Information Technology (accounting for 21.0% of the domains),
+followed by Business/Economy (16.1%), Education (6.4%), and Adult
+(6.1%). As highlighted earlier, in general we observe the distribution is
+skewed towards higher ranks for most categories, showing how attacks
+generally target highly popular domains. Exceptions are categories with
+significant geographical components such as News and Media, Business
+and Economy, Cultural Institutions, and Real Estate, all of which show
+a more spread behavior. Table 5 shows the top 5 reported domains for
+the top 10 categories by total number of domains in the category. The
+table captures the diverse range of popularity of abused domains, e.g., 6
+domains in the Tranco top 1K and 7 domains with a rank larger than
+500,000.
+</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1185,14 +1289,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3744A4C2-A66F-440C-B54D-D3DC708D0F68}">
-  <dimension ref="A2:F30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:F33"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.21875" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1212,225 +1316,252 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="409.6">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="409.6">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="360">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="409.6">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="345.6">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="244.9">
+      <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="360" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
+    <row r="9" spans="1:6" ht="409.6">
+      <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="345.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="1" t="s">
+    <row r="10" spans="1:6" ht="409.6">
+      <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="409.6">
+      <c r="A11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="230.45">
+      <c r="A12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="409.6">
+      <c r="A13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="259.14999999999998">
+      <c r="A14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="409.6">
+      <c r="A15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="316.89999999999998">
+      <c r="A16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="409.6">
+      <c r="A17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="244.9">
+      <c r="A18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="409.6">
+      <c r="A19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="388.9">
+      <c r="A20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="273.60000000000002">
+      <c r="A21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="409.6">
+      <c r="A22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="409.6">
+      <c r="A23" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="409.6">
+      <c r="A24" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="409.6">
+      <c r="A25" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="244.9">
+      <c r="A26" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="409.6">
+      <c r="A27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="302.45">
+      <c r="A28" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="259.14999999999998">
+      <c r="A29" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="1" t="s">
+    </row>
+    <row r="30" spans="1:3" ht="409.6">
+      <c r="A30" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="388.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="273.60000000000002" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="302.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="C30" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="405">
+      <c r="A31" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="409.6">
+      <c r="A32" t="s">
+        <v>64</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="409.6">
+      <c r="A33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1441,12 +1572,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57F51F23-009B-48D6-9CD6-BE19603B5BD6}">
   <dimension ref="A2:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1472,15 +1603,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007F0296C2CFEAD045A902F434C0DF9237" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="701b44b22bf6e624608469f647e94a1f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5146d105-7d5f-496c-bd31-80ca7e72687a" xmlns:ns4="3de855c3-8ecd-4254-b07d-50bb50556e99" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="303f33d50a37d12282966a9866b75223" ns3:_="" ns4:_="">
     <xsd:import namespace="5146d105-7d5f-496c-bd31-80ca7e72687a"/>
@@ -1719,7 +1841,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_activity xmlns="5146d105-7d5f-496c-bd31-80ca7e72687a" xsi:nil="true"/>
@@ -1727,46 +1849,23 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACE9AC90-BA89-410A-B600-14200351DC12}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCB68E56-5034-4584-86B1-FE0A3A1547B7}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCB68E56-5034-4584-86B1-FE0A3A1547B7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5146d105-7d5f-496c-bd31-80ca7e72687a"/>
-    <ds:schemaRef ds:uri="3de855c3-8ecd-4254-b07d-50bb50556e99"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93A08990-164D-4746-AA33-F52EDACD1948}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93A08990-164D-4746-AA33-F52EDACD1948}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="5146d105-7d5f-496c-bd31-80ca7e72687a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="3de855c3-8ecd-4254-b07d-50bb50556e99"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACE9AC90-BA89-410A-B600-14200351DC12}"/>
 </file>
</xml_diff>

<commit_message>
Finish 100-row evaluation and export
</commit_message>
<xml_diff>
--- a/data_awal.xlsx
+++ b/data_awal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SKRIPSI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A910858-0B9B-466C-9530-8FF78C4E2159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E91AA4C-9325-4B8F-A08F-B7C757413B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9DD10947-EA4E-42EA-8B01-D1CA78034524}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="205">
   <si>
     <t>Pertanyaan</t>
   </si>
@@ -892,6 +892,1176 @@
   <si>
     <t>Explain the concept of abused domain categorization as discussed in the scientific article Web of Shadows: Investigating Malware Abuse of Internet Services</t>
   </si>
+  <si>
+    <t>The main contributions of this paper are summarized as follows:
+•
+We propose a new multi-layer and adaptive security model (MAS) for DTNs intending to improve data-sharing efficiency between any physical-virtual pair. To ensure effective anomaly detection, predictive analytics, and behavioural analytics while maintaining data privacy, MAS integrates transfer learning, differential privacy (DP), and long short-term memory network (LSTM) algorithms. This provides a comprehensive approach to detecting malicious behaviour within such a system.
+•
+We incorporate a zero-trust security framework where nodes are not trusted by default in the network. Every node attempting to gain access to network resources must undergo a cost-aware verification process following the formulated game theoretic approach.
+•
+We implement the MAS framework and demonstrate its ability to enhance security in DTNs. The results show that MAS can offer robust solutions against sophisticated threats, ensuring the integrity and security of DTNs.</t>
+  </si>
+  <si>
+    <t>what the main contribution based on file Artificial intelligence-driven security framework for internet of
+things-enhanced digital twin networks?</t>
+  </si>
+  <si>
+    <t>Chao Liu , Fulong Chen ∗, Taochun Wang , Chuanxin Zhao , Dong Xie , Peng Hu</t>
+  </si>
+  <si>
+    <t>Who are the authors of the scientific article ‘A secure and dynamic fusion addressing scheme for Internet of Vehicles scenarios’?</t>
+  </si>
+  <si>
+    <t>What the abstract from article A secure and dynamic fusion addressing scheme for Internet of Vehicles
+scenarios?</t>
+  </si>
+  <si>
+    <t>The extensive deployment of Internet of Things (IoT) nodes has led to the emergence of various novel
+application scenarios, one of which is the Internet of Vehicles (IoV). Prior to efficacious data communication,
+IoT nodes must initially be equipped with a globally distinctive IPv6 address. Nevertheless, resource constraints
+and security vulnerabilities impose significant challenges to the addressing process. Existing addressing
+paradigms have been incapable of simultaneously meeting the requirements for security, scalability of the
+routing communication network, and address privacy protection of the terminal node. Consequently, they are
+not appropriate for utilization in IoV scenarios. To address these issues, this paper formulates a network model
+combining a static backbone network and a dynamic mobile network based on the characteristics of the IoV
+scenarios and designs a secure and dynamic fusion addressing scheme (SD-FAC). In SD-FAC, the backbone
+nodes utilize a lightweight security-enhanced neighbor discovery protocol based on location information to
+effectuate address registration, resisting message forgery, modification, and replay attacks, enhancing the
+security of the routing communication network, while supporting network scalability and automatic route
+establishment. The mobile nodes employ the congruence class approach to pre-construct independent address
+spaces and promptly complete association addressing upon entering the backbone network area. We analyze
+the addressing performance of the overall network model from eight indicators. Experimental simulation results
+demonstrate that the addressing latency, resource overhead, and energy consumption of the mobile network
+are all superior to those of the relevant addressing schemes.</t>
+  </si>
+  <si>
+    <t>With the rapid development of Industrial Internet of Things (IIoT) technology, it has played a core role in
+promoting the intelligent transformation of manufacturing industry. However, the complexity and diversity of
+IIoT environment also bring serious network security challenges, especially frequent incidents such as data
+breaches and device tampering, which pose significant threats to industrial security. As a key means of
+addressing such threats, the effectiveness and credibility of digital forensics directly depend on the security and
+efficiency of identity authentication schemes. This article proposes a secure and lightweight multi factor
+authentication scheme based on chebyshev chaotic mapping to address the identity authentication challenge of
+digital forensics in IIoT. This scheme enhances the strength of identity authentication through a three-factor
+authentication mechanism, utilizes chebyshev chaotic mapping to achieve efficient key negotiation. This
+article comprehensively verifies the scheme using security proof, BAN logic and Scyther. The results show that
+the scheme can effectively resist various malicious attacks and has high security and reliability. Compared with
+existing schemes, the proposed scheme significantly reduces costs and improves authentication efficiency while
+meeting security requirements, providing strong security support for digital forensics in IIoT.</t>
+  </si>
+  <si>
+    <t>What the abstract based on article A secure and lightweight authentication scheme for digital forensics in
+industrial internet of things?</t>
+  </si>
+  <si>
+    <t>Based on the performance analysis and theoretical analysis presented in the article ‘A Secure Distributed Resolution Model for Industrial Internet Identifier Based on Ordered Multi-Group Signature’, describe the complexity analysis of OMGS?</t>
+  </si>
+  <si>
+    <t>First, we analyze the complexity of OMGS. Assume that the number of groups is m, 𝑇𝐸 represents the time of bilinear pairing, 𝑇𝐻 represents the time of hash calculation, 𝑇𝐼𝑁𝑉 represents the time of inverse operation, 𝑇𝑀𝑈𝐿 represents the time of multiplication operations on the curve, 𝑇𝑀𝑂𝐷 represents the time of modular operations, and 𝑇𝐴𝐷𝐷represents the time of addition operations on the curve. We compare our algorithm with the group signature algorithms of lu [28] and gong [29] in terms of computational overhead.
+Table 2 is the comparison result of our algorithm with the group sig-nature algorithms of [28,29]. It shows the performance of signature and verification affected by the number of groups. The algorithm of [28] contains many operations of bilinear pairing, so the consumption of its algorithm is significantly greater than that of [29] and ours. The consumption of [29] is similar to ours. However, when a group member exits the group, [29] needs to regenerate keys for all users in the system, which has problems with system scalability.</t>
+  </si>
+  <si>
+    <t>Considering the aforementioned system model and security require-ments, our design goal is to develop a secure and reliable data sharing scheme for vehicular networks. Therefore, the following two objectives should be achieved:
+The proposed scheme must meet security requirements. If the scheme fails to satisfy these security criteria, unauthorized users may gain access to vehicle privacy information, including personalized data and spatiotemporal information. Due to privacy concerns, vehicles may not be able to provide sufficient data to support the development of vehicular network applications. Additionally, if RSUs or CSs illegally inject or tamper with data, it could render the data unreliable, leading to incorrect decision-making in vehicular network applications and posing a threat to traffic safety.
+The proposed scheme should ensure high efficiency. With the advance-ment of CPU and communication technologies, computational nodes in the network possess improved computing and communication perfor-mance. However, in applications based on vehicular network data shar-ing, a large number of sensing nodes need to upload data. At the same time, RSUs, as edge computing units, must process data in a timely manner to ensure that upper-layer applications can quickly provide services to users, especially in vehicular network applications related to user safety. Therefore, the scheme requires high computational and communication efficiency.</t>
+  </si>
+  <si>
+    <t>what is Design goals based on article Blockchain-cloud-based secure data sharing scheme with privacy
+preservation for Internet of vehicles</t>
+  </si>
+  <si>
+    <t>Existing trust management approaches have been observed to em-ploy various metrics to assess and quantify trust values.
+•
+Reputation-based metrics: The evaluator nodes’ recommenda-tions to the target nodes are the basis for calculating the trust value [11]. The shared recommendations are then disseminated throughout the network. The trust value will be heavily influ-enced based on the predominant recommendations, as this metric considers the global feedback received from the whole network.
+•
+Knowledge-based metrics: This metric allows for the identifica-tion of selfish nodes in the network by assessing trust based on direct or previous interactions a node has had with another node [10].
+•
+Expectation-based metrics: This metric involves a node assessing another node’s trustworthiness based on its anticipated behavior. In the absence of previous communication history, this may rely on a node’s previous interactions, recommendations, or initial forecast [11].
+•
+Node-properties-based metrics: Trust calculations primarily use node properties such as speed, direction, and resource availability to determine proximity and formulate the trust formula.
+•
+Environmental-factors-based metrics: This metric considers envi-ronmental factors such as network density and topology.
+•
+Proximity-based metrics: This metric uses main proximity param-eters like time, location, and distance to calculate trust in the IoV network.</t>
+  </si>
+  <si>
+    <t>Describe Trust metrics based on article Blockchain-based trust management systems in the Internet of Vehicles: A
+comprehensive survey</t>
+  </si>
+  <si>
+    <t>Smart contracts [36] are tools for structuring rules in
+programming code, registered in a DLT, such as Blockchain.
+The main objective of smart contracts is to automate the
+execution of rules and clauses, in addition to allowing those
+involved to monitor the execution process of each clause.
+Smart contracts work in such a way that, when a predetermined
+event occurs, another predetermined action will
+automatically occur, securely, and immutably. In addition,
+they are executed without the need for human action, since
+the code itself verifies each step, seeking to fulfill what was
+assigned. In practical terms, the smart contract “code” is
+compiled, generating an Application Binary Interface (ABI),
+which is recorded in a DLT as a transaction. Thus, each
+node that has access to the records can interact with this
+interface, executing smart contract methods. Because they
+run from DLT, smart contracts offer a higher level of security
+since they cannot be changed at run-time (a.k.a. deterministic
+execution). The most consolidate platform for smart
+contracts is the Ethereum[37] network. Ethereum nodes run
+the Ethereum Virtual Machine (EVM) that can run smart
+contracts implemented with the Solidity[38] programming
+language [39, 40].</t>
+  </si>
+  <si>
+    <t>what is Smart Contracts based on journal Coldnet: Vaccine Logistics Tracking by Integrating the Internet of
+Things and Smart Contracts: An Immutable and Reliable Approach</t>
+  </si>
+  <si>
+    <t>From the scenarios posed in the previous section, critical vulnerabilities and risks associated with unauthorized
+access, data manipulation, and communication security were highlighted. By analysing these findings,
+comprehensive insights into the challenges faced by agricultural systems are provided, and recommendations for
+strengthening cybersecurity measures through the integration of traditional approaches and innovative ZT principles
+can be suggested, as listed next:
+• Physical Access Vulnerability: by addressing the vulnerability of the VineInspector device to unauthorized
+physical access, the lack of robust physical security measures, such as locks and alarms were identified as main
+issues, potentially compromising the integrity devices operability. Recommendations emphasize the
+implementation of physical access controls, surveillance cameras – eventually, with some intelligence to
+recognize intrusion –, and continuous verification to mitigate the risk of unauthorized access. Furthermore, Zero
+Trust principles advocate for dynamic access control policies and remote device wiping capabilities to enhance
+security in the event of a breach.
+• Data Manipulation Risk: by exploring the risks associated with data manipulation within agricultural systems, the
+importance of ensuring the integrity of sensor data is underscored, to support reliable decision-making processes.
+Traditional cybersecurity measures, such as digital signatures and encryption, are recommended to protect against
+unauthorized data manipulation. Additionally, Zero Trust principles advocate for network segmentation and
+continuous verification to prevent malicious actors from corrupting reading in sensors.
+• Communication Security Concerns: the security challenges related to communication between the VineInspector
+device and the mySense platform, allowed to highlight the importance of securing data transmissions to preserve
+data integrity and reliability. Recommendations include implementing encrypted transmissions, multi-factor
+authentication, and regular security audits to mitigate communication security risks. Furthermore, Zero Trust
+principles emphasize the need for dynamic access control policies, network segmentation, and continuous
+verification to enhance the security of data communication channels.
+In summary, resorting to the previous analysis made focusing the VineInspector susceptibility to several forms of
+attack, the complexity of cybersecurity challenges in PA are underscored and the importance of adopting a holistic
+approach to security is promoted. By integrating traditional cybersecurity measures with Zero Trust principles,
+organizations can better protect critical assets and ensure the resilience and trustworthiness of agricultural
+operations. Through comprehensive security strategies, agricultural systems can effectively mitigate cybersecurity
+risks and maintain the integrity of agricultural data.</t>
+  </si>
+  <si>
+    <t>what discussion of the result based on journal Conventional and Zero Trust Security Measures for Precision
+Agriculture Devices: the mySense’s VineInspector Case-study?</t>
+  </si>
+  <si>
+    <t>IoT applications often involve the trans-mission of sensitive data, such as health information, locationdata, and industrial metrics. Ensuring end-to-end privacy insuch environments is critical, especially when sensor nodesare physically exposed and susceptible to tampering or com-promise. Lightweight encryption and secure data transmissionprotocols must be integrated into IoT systems to protect againstunauthorized access while preserving device efficiency.</t>
+  </si>
+  <si>
+    <t>What is Privacy and Data Security based on journal Current research on Internet of Things (IoT) security protocols: A survey</t>
+  </si>
+  <si>
+    <t>•
+User authentication.
+•
+User anonymity.
+•
+Reparability.
+•
+Secure session key establishment.
+•
+GWN secret key/parameter must be secure.
+•
+User-friendly registration phase.
+•
+Reduces the transmission overhead between the sensor nodes.
+•
+Mutual authentication between the user and Base Station(BSs).
+•
+Mutual authentication between the BS and sensor node.
+•
+Secure and user-friendly password change phase.
+•
+Authentication and key-agreement protocol should be suitable forresource-constrained devices</t>
+  </si>
+  <si>
+    <t>What is the critical features are essential in WSNs security protocols based on journal Current research on Internet of Things (IoT) security protocols: A survey?</t>
+  </si>
+  <si>
+    <t>The IoT refers to a network of interrelated physical devices that
+interact and exchange data with each other through the Internet. The
+IoT comprises multiple components, such as sensors, actuators, software
+or network protocols, and other wireless electronic technologies.
+These components aim to create an all-in-one, intelligent network
+where devices can work together to improve efficiency, automation,
+and overall functionality (Khanna and Kaur, 2020). The IoT devices
+are used in various applications across different industries, including
+industrial plants, health-care IoT, battlefield surveillance, smart home
+monitoring, traffic monitoring, etc. (Laghari et al., 2021; Schiller et al.,
+2022). IoT devices use multiple heterogeneous devices and components
+to perform various surveillance and monitoring operations. Fig. 1 shows
+the IoT network model. The IoT comprises various components and
+network protocols to ensure end-to-end services. Some of the critical
+components are as follows:
+• Wireless Sensor Nodes
+• Actuators
+• Gateway Nodes
+• Communication network protocols
+• Security protocols</t>
+  </si>
+  <si>
+    <t xml:space="preserve">describe IoT architecture based on journal Current research on Internet of Things (IoT) security protocols: A survey
+</t>
+  </si>
+  <si>
+    <t>In this manuscript, we conducted a comprehensive cryptanalysis
+and survey of security protocols within the IoT ecosystem. We aimed
+to highlight the current challenges and opportunities in IoT security
+applications, providing a valuable reference for emerging researchers
+by reviewing reputable research articles. We specifically analyzed three
+security protocols—those by Guo et al. (2019), Alzahrani et al. (2021),
+and Lu et al. (2019)—evaluating their computational costs and security
+features. Through this analysis, we identified several vulnerabilities,
+including susceptibility to offline device attacks, stolen user verifier
+attacks, and issues related to perfect forward secrecy. Moreover, we
+discussed the challenges and opportunities in the field of IoT security
+protocols, emphasizing the need for tailored security solutions suitable
+for low-power Wireless Sensor Networks (WSNs). Our findings serve as
+a foundation for future research directions in authentication and key
+agreement protocols, guided by the evolving threat landscape in IoT
+environments.</t>
+  </si>
+  <si>
+    <t>What conclusions are presented in Current research on Internet of Things (IoT) security protocols: A survey?</t>
+  </si>
+  <si>
+    <t>To reveal the bottleneck of the security protocols, we make acomprehensive comparison with the security features. The details ofthe security features are displayed in
+Table 3. Here, we have examinedsecurity protocols with a range of features and assaults, including re-play attacks, man-in-the-middle attacks, physical attacks, loss of deviceattacks, user anonymity, forward secrecy, and sensor anonymity.It is noted that complete forward secrecy, password guessing, anduser anonymity are absent from the security protocol. It is also evidentthat the security protocols do not handle sensor nodes’ physical secu-rity. We also observed that the security protocol requires a high compu-tation overhead, which reduces the lifespan of the low-powered sensornodes. The lightweight authentication protocol’s main objective is toprovide end-to-end security with limited computation overhead andprevent the unauthorized access of attackers. In the present manuscript,we perform the cryptanalysis of three security protocols in the IoTecosystem.6. Discussion</t>
+  </si>
+  <si>
+    <t>Describe about Security features on journal Current research on Internet of Things (IoT) security protocols: A survey?</t>
+  </si>
+  <si>
+    <t>The protection of user privacy and confidentiality, the guaranteeof user anonymity, and the assurance of service accessibility are thethree main goals of authentication and key agreement protocols inIoT environments. It is well-recognized that authentication and keyagreement protocols provide security trust management and ensurethe availability of legitimate users’ resources. The security protocolsalso prevent cyber attacks by malicious users or nodes. Research oninexpensive and lightweight encryption methods for low-power sensornodes is another area of attention for security protocols.
+The computational cost of the security mechanisms for the Internetof Things environment will be covered in this subsection.Table
+2compares the computing costs of the three distinct security protocols.The security protocols use multiple operations during login, authentica-tion, and verification of legitimate users. These operations are modular,exponentiations, session key generation, and hash operations. All theseoperations required the computation overhead on the gateway node,sensor node, and user devices. Here, we analyze the security protocolsbased on the overall computation overhead with all the phases.</t>
+  </si>
+  <si>
+    <t>based on journal Current research on Internet of Things (IoT) security protocols: A survey describe Computation cost on Performance analysis section</t>
+  </si>
+  <si>
+    <t>Here, we discuss the key ethical concerns that belong to the IoD
+communication. It includes data sovereignty problems, because drones
+operate across different borders may be from different countries or
+states of a country, which potentially violates local laws (for example,
+the laws on data storage and its processing). Another potential
+challenge is ‘‘General Data Protection Regulation (GDPR)’’. It is the
+European Union (EU) law that regulates how organizations handle
+personal data [7]. It complies with the risk of unauthorized personal
+data collection and excessive data processing [8]. IoD communication
+also faces concerns of data privacy, surveillance and accountability.
+To address these issues and challenges, some of the strategies, such
+as data localization, privacy-by-design, use of strong encryption and
+global regulatory standards, are necessarily needed [9].</t>
+  </si>
+  <si>
+    <t>what is Potential ethical concerns belong to IoD communication based on journal Designing secure blockchain-based authentication and key management
+mechanism for Internet of Drones applications</t>
+  </si>
+  <si>
+    <t>Security solutions are essential for safeguarding the data and devices,
+such as drones and servers, within IoD networks. A reliable
+blockchain-enabled authentication and key management mechanism
+for various IoD applications (BAKMM-IoD) was introduced. BAKMMIoD
+has been demonstrated to be secure against numerous potential
+threats through comprehensive security study and formal verification
+with the widely recognized Scyther tool. BAKMM-IoD outperforms
+other comparable current mechanisms regarding communication cost,
+calculation cost, and attributes of security and functionality. At the end,
+a practical implementation of BAKMM-IoD is subsequently shown to
+illustrate its applicability in real-world scenarios and highlight its effect
+on key performance metrics.
+In the future, we intend to provide machine learning/deep learningbased
+big data analytics phase in the presented scheme for the real-time
+data analysis of the received data. We have plan to provide a testbed
+implementation for the presented scheme. The post-quantum cryptography
+(PQC)-based security primitives can also be incorporated in the
+design of the presented scheme to make it more secure especially for
+the era of quantum cryptography.</t>
+  </si>
+  <si>
+    <t>what is conclusion of Designing secure blockchain-based authentication and key management
+mechanism for Internet of Drones applications</t>
+  </si>
+  <si>
+    <t>Following are the main objectieves of the proposed study:
+•
+In the suggested study, a novel and special framework called Dip- DARK, which stands for Dipper Throated Optimization integrated Deep Activation based Runge Kutta Classifier, is created for pro
+tecting the HetIoT network from hazardous intruders.
+•
+For system installation and validation, some of the well-known and most recent intrusion datasets, including CIC-DDoS 2019, ToN-IoT, Edge-IIoT, and In-SDN, have been employed.
+•
+Then, the most pertinent features are optimally chosen using the Dipper Throated Optimization (DipTO) model, an intelligent opti
+mization tool, to efficiently reduce the size of the dataset.
+•
+As a result, using the set of optimized features, the Deep Activation based Runge Kutta (DARK) classifier was able to predict the type of intrusion with accuracy.
+•
+Additionally, the proposed Dip-DARK model’s intrusion detection findings are tested and compared with current state-of-the-art model techniques utilizing a range of performance metrics.</t>
+  </si>
+  <si>
+    <t>what the objective of journal Dip-DARK: A smart and innovative classifier for enhanced intrusion
+detection and security in heterogeneous IoT networks</t>
+  </si>
+  <si>
+    <t>Presently, significant research works focused on the design and development of security methods for protecting
+Heterogeneous Internet of Things (HetIoT) networks. Yet, the conventional approaches suffer with the problems
+of high processing time, lower accuracy, increased system designing complexity, and reduced efficiency.
+Therefore, in the proposed study, a novel and unique framework known as Dip-DARK—Dipper Throated Optimization
+integrated Deep Activation based Runge Kutta Classifier—is developed to safeguard the HetIoT network
+from potentially dangerous intrusions. Some of the well-known and most recent intrusion datasets, including as
+CIC-DDoS 2019, ToN-IoT, Edge-IIoT, and In-SDN, have been used for system development and validation. The
+proposed model is validated and tested by using these datasets. Then, to effectively shrink the dataset, the most
+important features are best selected using the Dipper Throated Optimization (DipTO) model, an intelligent
+optimization method. As a result, the Deep Activation based Runge Kutta (DARK) classifier was able to precisely
+predict the type of intrusion using the set of optimized features. Additionally, using a variety of performance
+measures, the proposed Dip-DARK model’s intrusion detection findings are evaluated and contrasted with current
+state-of-the-art model methodologies</t>
+  </si>
+  <si>
+    <t>what is abstract based on journal Dip-DARK: A smart and innovative classifier for enhanced intrusion
+detection and security in heterogeneous IoT networks</t>
+  </si>
+  <si>
+    <t>The application of ICN in IoT is an evolving research field. ICN
+enhances the availability of IoT data through distributed data caching
+while introducing new challenges in the authentication field. Xue
+et al. [44] explored the impacts of EDOS attacks in CP-ABE encrypted
+cloud systems. Meanwhile, Salvador et al. [45] introduced an innovative
+architecture merging CP-ABE’s adaptability with symmetric key
+encryption’s efficiency, aiming for secure data transfer and privacy.
+While current research demonstrates significant advancements in integrating
+CP-ABE, blockchain, and ICN within IoT environments to
+enhance security, efficiency, and scalability, a critical need remains
+for further exploration into optimized, cohesive solutions that address
+IIoT systems’ rapidly evolving and specific challenges. Table 1 summarizes
+the key features of the existing studies discussed in this section,
+providing a clear comparison with the proposed framework.</t>
+  </si>
+  <si>
+    <t>what is ICN with IoT based on journal  DPS-IIoT: Non-interactive zero-knowledge proof-inspired access control
+towards information-centric Industrial Internet of Things</t>
+  </si>
+  <si>
+    <t>The advancements in 5G/6G communication technologies have enabled the rapid development and expanded
+application of the Industrial Internet of Things (IIoT). However, the limitations of traditional host-centric
+networks are becoming increasingly evident, especially in meeting the growing demands of the IIoT for
+higher data speeds, enhanced privacy protections, and improved resilience to disruptions. In this work, we
+present the ZK-CP-ABE algorithm, a novel security framework designed to enhance security and efficiency in
+distributing content within the IIoT. By integrating a non-interactive zero-knowledge proof (ZKP) protocol
+for user authentication and data validation into the existing Ciphertext-Policy Attribute-Based Encryption
+(CP-ABE), the ZK-CP-ABE algorithm substantially improves privacy protections while efficiently managing
+bandwidth usage. Furthermore, we propose the Distributed Publish-Subscribe Industrial Internet of Things
+(DPS-IIoT) system, which uses Hyperledger Fabric blockchain technology to deploy access policies and ensure
+the integrity of ZKP from tampering and cyber-attacks, thus enhancing the security and reliability of IIoT
+networks. To validate the effectiveness of our approach, extensive experiments were conducted, demonstrating
+that the proposed ZK-CP-ABE algorithm significantly reduces bandwidth consumption, while maintaining
+robust security against unauthorized access. Experimental evaluation shows that the ZK-CP-ABE algorithm
+and DPS-IIoT system significantly enhance bandwidth efficiency and overall throughput in IIoT environments.</t>
+  </si>
+  <si>
+    <t>what is abstract based on journal DPS-IIoT: Non-interactive zero-knowledge proof-inspired access control
+towards information-centric Industrial Internet of Things</t>
+  </si>
+  <si>
+    <t>In this work, a comprehensive set of experimental configurations
+is carefully designed to demonstrate the system’s ability to accommodate
+large volumes of traffic while minimizing bandwidth usage. The
+blockchain is implemented using Hyperledger Fabric to store access
+control policies and validate user requests via smart contracts. For
+experimental evaluation, the hardware configuration comprises two
+computer servers: the first equipped with a 3.60 GHz i7-7700 CPU
+and 8 GB of RAM, and the second furnished with an i7-7500U CPU
+at 2.90 GHz coupled with 16 GB RAM. Additional apparatus includes a
+1.5 GHz Raspberry Pi with 4 GB RAM, powered by an ARM A72 CPU.
+The dataset used in the experiments is simulated to model typical IIoT
+traffic scenarios, including data from smart manufacturing, healthcare,
+and industrial sensors.</t>
+  </si>
+  <si>
+    <t>describe Experimental settings on journal DPS-IIoT: Non-interactive zero-knowledge proof-inspired access control
+towards information-centric Industrial Internet of Things</t>
+  </si>
+  <si>
+    <t>The blockchain system is deployed on 𝑃 𝐶1 using multiple virtual
+machines, each equipped with a customized chain code (smart contract).
+To emulate a realistic IC-IoT environment, MQTT is adopted as
+the communication protocol, and the broker, EMQ, is deployed on 𝑃 𝐶1
+within a Docker container. On 𝑃 𝐶2, subscriber and publisher clients
+are implemented to interact via the MQTT protocol, with each client
+possessing the ability to invoke the chain code within the blockchain.
+Additionally, a client is deployed on a Raspberry Pi to emulate a device,
+programmed to periodically upload data and maintain transmission
+in adherence to the MQTT protocol. The results shown in Fig. 6
+capture the average response time as the number of concurrent clients
+increases. The simulation utilizes MQTT based architecture, EMQ agent
+deployed on Docker, and smart contract interaction.
+To assess the system’s throughput capabilities in a distributed
+context, experiments were conducted simulating various counts (denoted
+as 𝑁) of concurrent subscriber/publisher clients accessing the
+blockchain system over a predefined duration to evaluate the average
+response time. Specifically, 𝑁 is varied within the set {50, 100,…, 500}.
+In the context of CP-ABE, the attribute count for testing is consistently
+set at 𝐾 = 50, and the data block size is fixed at 𝑆 = 512𝐾 𝐵. The results
+are shown in Fig. 6(c).</t>
+  </si>
+  <si>
+    <t>explain System performance evaluation based on journal DPS-IIoT: Non-interactive zero-knowledge proof-inspired access control
+towards information-centric Industrial Internet of Things</t>
+  </si>
+  <si>
+    <t>The implementation of CP-ABE in IIoT primarily aims to enhance
+efficiency in key management, access control structures, and algorithmic
+complexity. For instance, Li et al. [30] introduced a Distributed
+Publisher-Driven secure data-sharing system for IC-IoT, reducing
+the communication overhead in CP-ABE systems. In another
+study, Li et al. [31] proposed a verifiable flexible data sharing (VFDS)
+mechanism, combining CP-ABE with identity-based signature (IBS)
+for distributed authentication in big-data sharing environments. Zhao
+et al. [32] focused on attribute revocation, proposing an outsourced
+CP-ABE scheme that maintains fixed ciphertext and key sizes. Zhang
+et al. [33] propose BCAE, a blockchain-based cross-domain authentication
+scheme for edge computing, enhancing secure identity verification
+and efficient key agreement for IoT devices through digital certificates,
+digital signatures, and blockchain technology. Khan et al. [34]
+addressed the limitations of traditional consensus mechanisms in private
+blockchains by proposing B-LPoET, a scalable and efficient multithreaded
+approach. This innovative consensus strategy informs our
+methodology for integrating blockchain with CP-ABE to optimize performance
+in IIoT contexts. Vanga et al. [35] suggested an RSA-based
+CP-ABE scheme with constant key and ciphertext size. Finally, Hao
+et al. [36] developed a CP-ABE system supporting entirely hidden
+attribute-based access policies using a garbled Bloom filter.</t>
+  </si>
+  <si>
+    <t>explain about Attribute-based encryption with IoT based on journal  DPS-IIoT: Non-interactive zero-knowledge proof-inspired access control
+towards information-centric Industrial Internet of Things</t>
+  </si>
+  <si>
+    <t>This section uses the relatively mature automated protocol anal-ysis software Scyther to demonstrate the security of the proposed scheme. Scyther is used to analyze the security of registration phase and message authentication phase of the proposed scheme. Users use the security policy definition language to write the authentication process of sending and receiving messages between roles in Scyther. Scyther detects and analyzes the security attributes defined by the user. If it searches for an attack path, it displays the attack process in a graphical way. The declared events are used to define the security attributes to be implemented by the protocol, mainly including Secret, Alive, Weak-agree, Nisynch, and Niagree. Secret means that the parameter item is confidential and secure, Alive means that the entity is active during the operation of the protocol, and Nisynch, Niagree, and Weakagree are mainly used to detect whether the protocol can resist attacks such as replay attacks, tampering attacks, and eavesdropping attacks. Ref. [55] gives detailed definitions. Figs. 4and5 show the verification results. The results show that the declared security attributes are true and no attack path is found within the limited query range, that is, the proposed scheme is secure.</t>
+  </si>
+  <si>
+    <t>what is Formal security verification using scyther based on journal Edge-assisted lightweight message authentication for Industrial Internet of
+Things?</t>
+  </si>
+  <si>
+    <t>In the Industrial Internet of Things (IIoT) environment, smart devices face the risk of data security and privacy
+leakage when sharing data. Message authentication is a crucial mechanism for ensuring data security. However,
+existing authentication schemes still encounter various challenges in privacy protection and efficiency. To
+address these issues, this paper proposes an edge-assisted lightweight message authentication scheme, where
+edge servers assist smart devices in data authentication, thereby reducing their computational burden.
+Specifically, dynamic pseudonym updates enable anonymous authentication and unlinkability, while dynamic
+public–private key pairs enhance key security, effectively safeguarding the data privacy of smart devices.
+To tackle efficiency bottlenecks, a lightweight message authentication algorithm and a batch authentication
+algorithm leveraging edge computing are designed to improve authentication efficiency. Security analysis and
+theoretical proof demonstrate the proposed scheme’s significant advantages in privacy protection. Performance
+evaluations further validate its low computational cost and reasonable communication overhead.</t>
+  </si>
+  <si>
+    <t>what is abstract from journal Edge-assisted lightweight message authentication for Industrial Internet of
+Things</t>
+  </si>
+  <si>
+    <t>what is Certificate-less public key encryption from journal Edge-assisted lightweight message authentication for Industrial Internet of
+Things?</t>
+  </si>
+  <si>
+    <t>A one-way hash function takes an input of arbitrary length and produces a fixed-length binary output. For example, H(x) = y, where 𝑥 is the input data and 𝑦 is the hash value, with the mapping rule known as the hash algorithm. Hash functions possess the following main characteristics:
+•
+Efficiency. As they can compute the hash value of a message effectively;
+•
+It is designed to be computational hard to derive the original message from its hash value;
+•
+It is challenging to find another message that will produce the same hash value, which is called a collision.</t>
+  </si>
+  <si>
+    <t>explain hash function on journal Edge-assisted lightweight message authentication for Industrial Internet of
+Things</t>
+  </si>
+  <si>
+    <t>In the message authentication process of SDs in IIoT, various security
+and privacy issues pose threats to both the overall system security
+and the privacy of SDs. First, KGC within the IIoT system may be
+vulnerable to external attacks, making it inherently untrustworthy. If
+KGC is responsible for managing the private keys of SDs within the
+system, there is a risk of key leakage, which could severely compromise
+both the privacy of SDs and the security of the entire system. To
+mitigate this risk, the proposed scheme adopts CL-PKC to eliminate
+key escrow. Secondly, during message authentication, if the real identity
+of a SD is exposed on the network, identity information may be
+leaked. Therefore, pseudonyms must be employed in message authentication
+to conceal real identities. Additionally, when the same SD
+sends multiple messages, a malicious recipient could analyze the traffic
+and extract sensitive information. To address this issue, the proposed
+scheme dynamically updates pseudonyms and private keys to ensure
+message unlinkability. This scheme does not consider physical attacks
+on devices, such as side-channel attacks.</t>
+  </si>
+  <si>
+    <t>what is Security and privacy threats based on journal Edge-assisted lightweight message authentication for Industrial Internet of
+Things</t>
+  </si>
+  <si>
+    <t>what Formal security verification using scyther from journal Edge-assisted lightweight message authentication for Industrial Internet of
+Things</t>
+  </si>
+  <si>
+    <t>This paper proposes an anonymous and unlinkable message authentication
+scheme which is suitable for IIoT scenarios. The main goal
+of this scheme is to meet the security and efficiency requirements of
+IIoT message authentication. Specifically, we design an edge-assisted
+lightweight message authentication framework to achieve anonymity
+and unlinkability of message authentication. Then a lightweight message
+authentication algorithm and a batch authentication algorithm
+were designed. Detailed security proof and analysis show that the
+proposed scheme can resist various attacks. In addition, comparisons
+with related schemes show that the proposed scheme is lightweight in
+terms of computational and communication overheads, and is suitable
+for resource-constrained industrial IoT devices. In the future, we will
+design secure and efficient message authentication schemes for mobile
+smart devices for IIoT</t>
+  </si>
+  <si>
+    <t>what Conclusion from paper Edge-assisted lightweight message authentication for Industrial Internet of
+Things</t>
+  </si>
+  <si>
+    <t>This section analyzes the communication overhead of the proposed
+scheme in the message authentication phase and compares it with the
+communication cost of other comparative schemes. In order to analyze
+the communication cost, the length of the elements in 𝐺𝑖 is set to 128
+bytes, the length of the elements in 𝑍∗
+𝑞 is set to 20 bytes, the length of
+𝑅𝐼𝐷 is set to 16 bytes, the length of 𝑚 is set to 32 bytes, and the length
+of 𝑡 is set to 2 bytes. Table 7 lists the comparison of the communication
+cost of SD in the message authentication phase with other schemes,
+and Fig. 9 shows a more intuitive result. It can be seen from Table
+7 and Fig. 9 that without adding the update process (Our(WU)), the
+communication overhead of the proposed scheme is the same as [43]
+and lower than the other five schemes. When the update process is
+added, the communication overhead of the proposed scheme is on par
+with [53] and slightly higher than that of other schemes. Adding the
+update process will inevitably increase the communication overhead
+of the scheme, but it can achieve the unlinkability of the message
+and further protect the identity privacy and data privacy of SD. Most
+other solutions do not implement the unlinkability of messages. Moreover,
+compared with [53], which do not implement this function, the
+proposed scheme still has lower communication overhead. Therefore,
+based on security considerations, the communication overhead of the
+proposed scheme is reasonable.</t>
+  </si>
+  <si>
+    <t>What is Communication overhead based on paper Edge-assisted lightweight message authentication for Industrial Internet of
+Things</t>
+  </si>
+  <si>
+    <t>also limited by some challenges that are planned to be overcome in the
+future. The proposed model’s graph-based architecture and multi-head
+attention mechanisms increase computational complexity. Additionally,
+handling large volumes of data in real-time may strain network
+bandwidth and storage, especially in high-density IoT settings. Although
+deploying the model on edge nodes alleviates these limitations, it requires
+sufficient infrastructure to support real-time processing and
+secure data aggregation. Future work aims to refine the model for
+deployment in edge and gateway environments, potentially through
+model compression techniques such as pruning, quantization, and
+knowledge distillation. Furthermore, combining EIW-AGTrans with
+adaptive sampling strategies could reduce the volume of data processed
+in real-time, targeting high-risk periods or specific network segments.
+Through these optimizations, EIW-AGTrans could provide robust
+security in IoT networks while meeting the efficiency requirements of
+modern IoT deployments. Further, we aimed to test the model on realworld
+datasets collected from live IoT networks as part of future work.</t>
+  </si>
+  <si>
+    <t>what is Limitations and future work based on paper Edge Implicit Weighting with graph transformers for robust intrusion
+detection in Internet of Things network?</t>
+  </si>
+  <si>
+    <t>In recent years, the Internet of Things devices have progressively deployed in various applications including
+smart cities, intelligent transportation, healthcare, and agriculture. However, this widespread adaptation of the
+Internet of Things networks has been vulnerable to several attacks. Lack of security protocols, unauthorized
+access, and improper device updates lead the Internet of Things environment to several attacks, which impact
+network security and confidentiality of users. This paper develops an innovative approach that integrates Edge
+Implicit Weighting and Aggregated Graph Transformer architecture for accurate and timely intrusion detection.
+The proposed technique aggregates information from both one-hop and two-hop neighbors to derive immediate
+and extended relational context thereby improving the detection of complex attacks. This approach designs an
+Edge Implicit Weighting mechanism that allows the model to prioritize structurally significant relationships and
+enhance the accuracy of attack detection. The multi-head attention mechanism is introduced to enhance the
+detection of relevant patterns even in highly variable traffic scenarios. Further, the proposed framework incorporates
+the Synthetic Minority Over-sampling Technique to generate synthetic samples of minority classes to
+reduce class imbalance problems and attain balanced detection performance across all classes. The performance
+of the proposed detection technique is analyzed using multiple datasets with standard evaluation parameters.
+The proposed technique achieves outstanding performance results including an accuracy of 98.87% and a recall
+of 98.36%. From this experimental validation, it’s clear that the proposed framework provides robust performance
+under diverse network conditions and handles imbalanced data effectively.</t>
+  </si>
+  <si>
+    <t>what is abstract from paper Edge Implicit Weighting with graph transformers for robust intrusion
+detection in Internet of Things network</t>
+  </si>
+  <si>
+    <t>Timely attack detection is significant for preventing IoT networks
+from distinct attacks. This study introduces a novel technique named
+EIW-AGTrans that combines the significance of EIW and AGTransformer
+for accurate intrusion detection in IoT networks. The EIW mechanism is
+utilized to prioritize critical connections in the graph by assigning
+weights based on relational significance. To capture both direct and
+indirect relationships, the AGTransformer aggregates information from
+both one-hop and two-hop neighbors and detects complex attack patterns
+effectively. The proposed EIW-AGTrans technique uses a multihead
+attention mechanism for processing high-dimensional data and
+making it suitable for real-time intrusion detection. This dual aggregation
+of EIW and AGTransformer allows the model to capture multi-stage
+and coordinated attacks that may not be detectable by existing works. In
+addition, the proposed EIW-AGTrans model incorporates the SMOTE
+technique to generate synthetic samples of minority classes to minimize data imbalance problems. Further, the comprehensive performance
+evaluation is conducted with several evaluation parameters on the ToNIoT,
+UNSW-NB15, CSE-CIC-IDS, and CCI-DarkNet datasets. The model’s
+performance on ToN-IoT, UNSW-NB15, CSE-CIC-IDS, and CCI-DarkNet
+datasets highlights its ability to maintain high accuracy, precision, and
+recall, even when faced with imbalanced data distributions. The proposed
+EIW-AGTrans framework attains 98.87% accuracy, 98.61% precision,
+98.36% recall, 98.25% specificity, 98.48% F1 score, 0.144% FPR,
+and 0.027% FNR. The experimental results are compared with existing
+IoT-based attack detection approaches namely GGCN, E-GraphSAGE,
+MQBHOA, FN-GNN, HAD-IDS, GTO-BSA, and AttackNet. From the
+experimental analysis, we confirm that the EIW-AGTrans approach is
+highly effective in detecting and classifying diverse attacks that affect
+IoT networks and also outperforms existing works.
+5.1. Limitations and future work
+Despite its benefits in attack detection, the EIW-AGTrans approach is
+also limited by some challenges that are planned to be overcome in the
+future. The proposed model’s graph-based architecture and multi-head
+attention mechanisms increase computational complexity. Additionally,
+handling large volumes of data in real-time may strain network
+bandwidth and storage, especially in high-density IoT settings. Although
+deploying the model on edge nodes alleviates these limitations, it requires
+sufficient infrastructure to support real-time processing and
+secure data aggregation. Future work aims to refine the model for
+deployment in edge and gateway environments, potentially through
+model compression techniques such as pruning, quantization, and
+knowledge distillation. Furthermore, combining EIW-AGTrans with
+adaptive sampling strategies could reduce the volume of data processed
+in real-time, targeting high-risk periods or specific network segments.
+Through these optimizations, EIW-AGTrans could provide robust
+security in IoT networks while meeting the efficiency requirements of
+modern IoT deployments. Further, we aimed to test the model on realworld
+datasets collected from live IoT networks as part of future work.</t>
+  </si>
+  <si>
+    <t>what is Conclusion based on paper Edge Implicit Weighting with graph transformers for robust intrusion
+detection in Internet of Things network</t>
+  </si>
+  <si>
+    <t>Despite the significant performance of existing works in attack detection, there exists a significant knowledge gap, particularly low detection accuracy, high computational complexity, high false alarm rate, overfitting, class imbalance, and data scarcity. These limitations affect the ability of existing works to obtain superior detection outcomes. This research gap highlights the need for adaptable, scalable, and context-aware IDS that efficiently processes IoT data while achieving balanced detection across all types of attacks. In this study, we design an EIW-AGTrans framework to tackle these gaps and provide excellent intrusion detection results. The AGTransformer model incorporates EIW, which prioritizes critical connections in the graph by assigning weights based on relational significance. This allows the model to focus on high-impact relationships, improving its sensitivity to interactions that may indicate malicious behavior, even in large networks. The model introduces an edge weighting mechanism that adjusts the importance of two-hop neighbors based on their connectivity strength with one-hop neighbors. This weighting helps prioritize structurally significant relationships, allowing the model to focus on interactions that may be indicative of attacks. To capture both direct and indirect relationships, the proposed model aggregates information from both one-hop and two-hop neighbors. This dual aggregation approach allows the model to capture multi-stage and coordinated attacks that may not be detectable by existing models. By leveraging multi-head attention, the proposed model is capable of examining network data from multiple perspectives, enhancing its ability to detect diverse attack patterns with low computational complexity. In addition, the model incorporates the SMOTE technique to generate synthetic samples of minority classes thereby reducing class imbalance issues.</t>
+  </si>
+  <si>
+    <t>What is Research gap from paper title Edge Implicit Weighting with graph transformers for robust intrusion
+detection in Internet of Things network</t>
+  </si>
+  <si>
+    <t>The recommendation system within cloud-integrated Internet of Vehicles (IoV) frameworks
+enhances user driving experiences by aggregating real-time telematics data from onboard
+terminals. To safeguard location-sensitive and other private data, vehicle owners encrypt their
+information prior to transmission. Consequently, the efficient utilization of such encrypted
+datasets emerges as a pivotal challenge. Although existing attribute-based encryption with
+keyword search (ABKS) schemes facilitate keyword retrieval over encrypted storage, their
+static trapdoors lack temporal constraints—enabling unrestricted search capabilities. This design
+flaw exposes a critical vulnerability: once user private keys are exposed, attackers can exploit
+perpetual trapdoors to compromise historical data privacy. To address this, we propose a
+novel cryptographic construct termed forward secure key policy attribute-based encryption with
+keyword search (FS-KP-ABKS). Our framework integrates temporal metadata into both ciphertexts
+and trapdoors, restricting cloud servers to accessing only those ciphertexts generated prior to
+the trapdoor’s associated secret key issuance time. We formally prove, within the standard
+cryptographic model, that FS-KP-ABKS achieves selective security against chosen-keyword attacks
+(SCKA). Comprehensive experimental evaluations further validate that our scheme’s unbounded
+attribute universe ensures scalable adaptability for IoV deployments, while its trapdoor generation
+and search mechanisms demonstrate superior computational efficiency.</t>
+  </si>
+  <si>
+    <t>what is abstract from paper Effective forward secure key policy attribute-based encryption
+with keyword search in recommendation system for Internet of
+vehicles</t>
+  </si>
+  <si>
+    <t>The following is a summary of this paper’s primary contributions:
+1)
+We introduce a novel cryptographic paradigm termed FS-KP-ABKS that unifies forward security, key-policy attribute-based encryption, and keyword search functionalities, which integrates temporal constraints into ABKS frameworks. This design mandates that trapdoors can only decrypt ciphertexts generated prior to their associated secret key’s issuance time, thereby confining server search operations to historical data and inherently protecting user privacy against post-compromise attacks.
+2)
+Using the techniques of 0-Encoding and 1-Encoding, we provide the first workable FS-KP-ABKS method in the prime order group and demonstrate that it guarantees selective protection for chosen-keyword attack scenarios within the standard cryptographic framework, assuming the hardness of the Modified 𝑞-2 problem.
+3)
+When compared to the related KP-ABKS schemes, the comprehensive performance demonstrates that our FS-KP-ABKS attains remarkable efficiency in trapdoor generation and search execution, demonstrating its applicability in the IoV system and its ability to support the dynamic addition of verifiable attributes due to the large universe.</t>
+  </si>
+  <si>
+    <t>what Contribution from paper Effective forward secure key policy attribute-based encryption
+with keyword search in recommendation system for Internet of
+vehicles</t>
+  </si>
+  <si>
+    <t>In practical cloud storage systems, servers typically permit continuous uploading of newly encrypted data. However, this function
+ality introduces a security vulnerability: the cloud server can exploit previously issued trapdoors to search through newly added data. Without forward security in Attribute-Based Keyword Search (ABKS), these legacy trapdoors may be misused during data addition, potentially compromising the confidentiality of freshly encrypted content. To achieve forward security, the system must ensure that historical trapdoors remain incapable of performing search operations on subsequently uploaded data until updated trapdoors are issued. Our proposed solution resolves this critical issue by implementing strict trapdoor expiration controls.</t>
+  </si>
+  <si>
+    <t>from Problem formulation what is Forward security based on paper Effective forward secure key policy attribute-based encryption
+with keyword search in recommendation system for Internet of
+vehicles</t>
+  </si>
+  <si>
+    <t>This paper presents a novel approach aimed at developing a secure secret key-sharing system optimized for resource-constrained
+Internet of Things (IoT) devices. Focusing on the MQTT protocol, the research endeavors to establish secure communication
+channels between IoT devices and brokers, thereby enhancing the overall security of MQTT-based IoT deployments. This research
+introduces a novel Dynamic Lightweight Authentication for MQTT (DLA-MQTT) mechanism designed to the unique needs of
+IoT devices operating under the MQTT protocol. The DLA-MQTT mechanism leverages an innovative lightweight Generalized
+Feedback Shift Register (GFSR)-based Pseudo-Random Number Generator (PRNG) to generate ephemeral keys, ensuring secure
+communication while addressing the limitations of computational power and energy resources. Through a detailed comparative
+analysis with existing cryptographic solutions, the DLA-MQTT mechanism demonstrates superior performance in terms of
+computational overhead, energy consumption, and execution time, while maintaining robust security against common attacks such
+as Man-in-the-Middle (MitM) and Denial of Service (DoS). he proposed algorithm’s adaptability and scalability are validated using
+the Cooja simulator, where simulated IoT networks are subjected to various threat scenarios. The results confirm the DLA-MQTT
+mechanism’s efficacy, showcasing a significant reduction in resource utilization without compromising the strength of the security
+provided.</t>
+  </si>
+  <si>
+    <t>what is abstract from paper Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>Current research predominantly focuses on static security protocols that, while effective in certain scenarios, do not
+adequately address the dynamic nature of IoT networks. These networks are characterized by frequent changes in
+device states, network topology, and evident threats. The existing security solutions often fall short in providing the
+flexibility and adaptability required to cope with these changes, especially in the context of MQTT, which is widely
+adopted for IoT communications due to its lightweight and efficient messaging system.</t>
+  </si>
+  <si>
+    <t>what is Dynamic Authentication for Resource-Constrained IoT Devices on paper Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>The DLA-MQTT mechanism is primarily composed of a set of algorithms, each of which is carefully crafted to
+perform particular functions within the security architecture. The fundamental algorithms of DLA-MQTT guarantee
+the resilience, effectiveness, and adjustability of the protocol to the resource-limited characteristics of IoT devices.
+The algorithms facilitate safe and effective device authentication and communication integrity by fusing cutting-edge
+cryptographic techniques with the low overhead requirements of MQTT.</t>
+  </si>
+  <si>
+    <t>what is Algorithm Design and Development based on paper Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>The main goal is to develop a lightweight secret key-sharing protocol for IoT devices, focusing on:
+• Designing an efficient key-sharing mechanism with minimal computational and energy demands.
+• Performing an in-depth security analysis to uncover and mitigate vulnerabilities in MQTT-based IoT
+networks.
+• Assessing the protocol’s computational efficiency, scalability, and security to ensure its real-world
+applicability.</t>
+  </si>
+  <si>
+    <t>what is Research Contributions based on paper Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>DLA-MQTT introduces several security enhancements aimed at fortifying MQTT communications against prevalent
+threats. The ephemeral nature of the session keys, coupled with the inclusion of nonce values in the handshake process,
+effectively counters the risk of replay attacks. Encryption of the authentication payload within the CONNECT message
+safeguards against eavesdropping and man-in-the-middle (MITM) attacks, ensuring that sensitive information remains
+confidential. Furthermore, the lightweight nature of the cryptographic operations is designed to mitigate the impact of
+resource exhaustion attacks, preserving device functionality even in adverse conditions</t>
+  </si>
+  <si>
+    <t>explain Security Enhancements based on paper Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>Furthermore, the integration of advanced cryptographic techniques, such as post-quantum cryptography and
+homomorphic encryption, into lightweight authentication mechanisms for MQTT has not been extensively explored.
+These techniques offer the potential for enhanced security against future threats but are often deemed too resourceintensive
+for constrained devices. Research is needed to adapt these advanced cryptographic concepts into practical,
+lightweight solutions suitable for MQTT-based IoT communications.</t>
+  </si>
+  <si>
+    <t>explain Integration of Advanced Cryptographic Techniques from paper Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>Inspired by the simplicity of the MQTT protocol, the handshake protocol in DLA-MQTT is designed to minimize the
+number of messages exchanged between the IoT device and the broker. This protocol leverages the existing MQTT
+connection process, embedding authentication within the CONNECT and CONNACK messages to avoid additional
+network overhead. DLA-MQTT incorporates a streamlined handshake protocol that is precisely designed to minimize
+the exchange overhead inherent in traditional authentication processes. This protocol is ingeniously embedded within
+the MQTT’s existing CONNECT and CONNACK message exchange framework, thereby leveraging the protocol’s
+inherent efficiency and reducing the need for additional network traffic</t>
+  </si>
+  <si>
+    <t>what is Minimalistic Handshake Protocol based on paper Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>DLA-MQTT introduces several security enhancements aimed at fortifying MQTT communications against prevalent
+threats. The ephemeral nature of the session keys, coupled with the inclusion of nonce values in the handshake process,
+effectively counters the risk of replay attacks. Encryption of the authentication payload within the CONNECT message
+safeguards against eavesdropping and man-in-the-middle (MITM) attacks, ensuring that sensitive information remains
+confidential. Furthermore, the lightweight nature of the cryptographic operations is designed to mitigate the impact of
+resource exhaustion attacks, preserving device functionality even in adverse conditions.</t>
+  </si>
+  <si>
+    <t>what is Security Enhancements based on paper Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>The conceptual framework of DLA-MQTT represents a significant advancement in securing MQTT-based IoT
+communications, specifically addressing the challenges posed by resource-constrained devices. Through its innovative
+components—ephemeral key generation, a minimalistic handshake protocol, and lightweight cryptographic hashes—
+DLA-MQTT achieves a delicate balance between security and efficiency. This framework enhances the security
+posture of IoT networks, also ensures that the operational integrity of IoT devices is maintained, paving the way for
+wider adoption and more resilient IoT ecosystems. The empirical evaluation, conducted under various operational
+scenarios, highlights the mechanism's superiority in terms of lower energy consumption, reduced computational
+overhead, and swift execution times, all while maintaining robust security against common threats such as Man-inthe-
+Middle (MitM) and Denial of Service (DoS) attacks. Despite its promising outcomes, the DLA-MQTT mechanism
+is subject to certain limitations that warrant consideration. Firstly, the 64-bit key size, while sufficient for current
+security needs and resource constraints, may need to be re-evaluated in the face of evolving computational capabilities
+and advanced cryptographic attacks. Future work should focus on the integration of emerging technologies such as
+blockchain, AI, and quantum-resistant cryptography to bolster the security of IoT devices and networks.</t>
+  </si>
+  <si>
+    <t>what is Conclusion and Future Work based on paper Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>who are the authors of the paper with tittle Enabling Robust Security in MQTT-Based IoT Networks with
+Dynamic Resource-Aware Key Sharing</t>
+  </si>
+  <si>
+    <t>Sharadadevi Kaganurmath, Nagaraj Cholli</t>
+  </si>
+  <si>
+    <t>The Data Logging phase of the DASM Framework plays a crucial role in maintaining transparency, accountability, and security within the metaverse ecosystem. In this phase, the Auditing System meticulously records all data interactions, ML predictions, user activities, and system responses, creating a comprehensive audit trail for forensic analysis and post-incident investigation.
+Data logging involves capturing and storing data in a structured format, ensuring its integrity, authenticity, and accessibility for future analysis. Cryptographic hashing algorithms, such as SHA-256, are com-monly used to generate unique fingerprints or hashes for data integrity verification. This process ensures that logged data remains tamper-proof and verifiable, safeguarding its evidentiary value in forensic investigations.
+Forensic analysis of logged data involves reconstructing incident timelines, identifying root causes, and attributing responsibilities in the event of security breaches or incidents. By tracing and analyzing data interactions, the Auditing System provides valuable insights for contin-uous improvement, refinement, and optimization of security measures within the metaverse ecosystem.
+The recorded data serves as a valuable resource for post-incident analysis, supporting continuous improvement and refinement of the DASM framework’s security measures.</t>
+  </si>
+  <si>
+    <t>what is Data logging and forensic analysis based on paper Enhancing IoT security and healthcare data protection in the metaverse: A
+Dynamic Adaptive Security Mechanism</t>
+  </si>
+  <si>
+    <t>The DASM framework holds significant potential for real-world
+applications in IoT and Metaverse environments. Its ability to accurately
+identify malicious traffic ensures robust protection for IoT-based
+healthcare systems, safeguarding critical patient data and operational
+integrity. In the Metaverse, where interconnected IoT devices play a
+pivotal role in creating immersive and secure environments, DASM
+can act as a foundational layer to ensure trustworthiness and data
+integrity. For instance, in real-time patient monitoring, DASM can
+quickly detect and respond to abnormal activities, mitigating potential
+security breaches while ensuring uninterrupted healthcare delivery.
+The DASM framework, underpinned by its adaptive and dynamic capabilities,
+presents a significant advancement in IoT healthcare security.
+By addressing its limitations and building on the insights gained from
+this study, future iterations of the framework can further strengthen the
+resilience and scalability of IoT systems in the Metaverse and beyond.</t>
+  </si>
+  <si>
+    <t>what is Real-world applications based on paper Enhancing IoT security and healthcare data protection in the metaverse: A
+Dynamic Adaptive Security Mechanism</t>
+  </si>
+  <si>
+    <t>In the rapidly evolving landscape of the Metaverse, the synergistic integration of the Internet of Things
+(IoT) and Digital Twins (DT) represents a revolutionary paradigm shift, seamlessly bridging the real and
+virtual worlds. While this innovative convergence offers unprecedented potential, it also exposes a broader
+spectrum of security vulnerabilities that challenge conventional approaches. This research aims to fortify
+the multifaceted ecosystem of the Metaverse, with a particular emphasis on securing IoT healthcare data.
+Ensuring the protection of health information within the extensive network of interconnected devices in the
+Metaverse is paramount. Addressing this critical need, we introduce the Dynamic Adaptive Security Mechanism
+(DASM), an advanced Artificial Intelligence (AI)-driven framework meticulously crafted to enhance security
+adaptively. DASM operates as a comprehensive and real-time defensive layer, continuously recalibrating its
+strategies to reinforce the security matrix for both IoT and Digital Twins. This study provides a detailed
+examination of the foundational architecture of DASM and its AI-driven adaptive processes. We elucidate
+its pivotal role in strengthening the security framework within the complex terrain of the Metaverse. Through
+rigorous testing and validation using the IoT healthcare security dataset, the Random Forest model emerges
+as the top performer, achieving near-perfect metrics, including a Matthews Correlation Coefficient (MCC) of
+0.9989 and superior Balanced Accuracy, while also offering reduced training and inference times compared to
+the LSTM model. Although the LSTM model demonstrates strong accuracy, the ensemble approach of Random
+Forest balances computational efficiency and performance. The DASM framework sets a new benchmark in
+IoT security, offering a scalable and effective solution with significant implications for the future of Metaverse
+applications.
+1.</t>
+  </si>
+  <si>
+    <t>what is abstract from paper Enhancing IoT security and healthcare data protection in the metaverse: A
+Dynamic Adaptive Security Mechanism</t>
+  </si>
+  <si>
+    <t>What are the implications of DASM’s architecture for future IoT security frameworks in the metaverse?</t>
+  </si>
+  <si>
+    <t>A thorough analysis of the literature highlights that while bloc-kchain and AI-driven techniques have been proposed for securing IoT systems in the Metaverse [23,29], there is limited research on holistic, adaptive frameworks that can operate across multiple sectors, including healthcare. The architecture of DASM introduces a dynamic, AI-powered security layer that continuously evolves in response to threats, a feature largely absent from current frameworks. This re-search question aims to explore the broader implications of DASM’s architecture for future IoT security systems, particularly in sectors like healthcare, smart cities, and industrial IoT. We aim to evaluate whether DASM can serve as a model for developing scalable and adaptable IoT security solutions in the Metaverse.</t>
+  </si>
+  <si>
+    <t>How can DASM enhance the privacy and security of healthcare data transmitted through IoT devices in the metaverse?</t>
+  </si>
+  <si>
+    <t>As highlighted in previous research [27], healthcare data is es-pecially vulnerable in IoT ecosystems due to the sensitive nature of personal health information. Existing frameworks, such as those using AES encryption for data protection have made strides in securing data but are often static and unable to handle dynamic threats in real-time. Drawing from these studies, this research question focuses on how DASM’s AI-driven adaptability can offer enhanced protection for healthcare data in the Metaverse, ensuring both data privacy and system integrity, even in the face of sophisticated cyber-attacks.</t>
+  </si>
+  <si>
+    <t>How does the proposed DASM framework compare to traditional security approaches in terms of adaptability and efficiency?</t>
+  </si>
+  <si>
+    <t>Traditional security systems for IoT networks often rely on pre-defined protocols and static rule-based systems [22]. However, these approaches fail to address the rapidly changing security needs of the Metaverse. By reviewing state-of-the-art frameworks, such as trust-based management systems for performance enhancement and SDN-based models for attack detection [21,22], we have identified a gap in the application of dynamic, AI-based security mechanisms. This research question aims to compare DASM with these traditional frame-works to evaluate its adaptability to emerging threats, its efficiency in response time, and its computational overhead. We hypothesize that DASM’s real-time adaptive processes will offer superior performance over static, rule-based methods.</t>
+  </si>
+  <si>
+    <t>How can the integration of IoT and digital twins in the metaverse be
+effectively secured against emerging threats?</t>
+  </si>
+  <si>
+    <t>Several studies have underscored the significant security vulnerabilities
+within IoT-enabled environments, particularly as these devices
+become increasingly interconnected in the Metaverse [20,21]. The
+current methods primarily rely on static, rule-based security measures
+that fail to account for the dynamic and evolving nature of threats in
+virtual environments. This research question seeks to explore how an
+adaptive security mechanism can effectively address these challenges
+by dynamically evolving in response to emerging threats, particularly
+in the healthcare sector, where data confidentiality and availability are
+critical.</t>
+  </si>
+  <si>
+    <t>What role can AI-driven frameworks, such as the Dynamic Adaptive
+Security Mechanism (DASM), play in securing IoT healthcare data within
+the metaverse?</t>
+  </si>
+  <si>
+    <t>The role of AI in cybersecurity is well-documented, with AI algorithms
+offering superior capabilities in detecting, predicting, and
+mitigating cyber threats [23,27]. However, there is limited exploration
+of AI’s role in safeguarding IoT healthcare systems specifically within
+the Metaverse, which presents unique challenges. Drawing inspiration
+from previous research on machine learning (ML) and deep learning
+(DL) for IoT security [28], this research question aims to examine how AI-driven frameworks, such as DASM, can enhance the security of IoT healthcare systems by continuously adapting to changing threat landscapes. Specifically, we are interested in exploring how DASM, with its real-time learning capabilities, can ensure the privacy and integrity of sensitive healthcare data</t>
+  </si>
+  <si>
+    <t>The Feedback Loop Initiation stage of the DASM Framework em-bodies the proactive and adaptive nature of its security mechanism. Malicious activities or security threats detected by ML-augmented Traf-fic Monitoring Systems serve as triggers for initiating corrective mea-sures in real-time. This feedback loop enables the system to respond swiftly and decisively to emerging threats, mitigating potential risks and vulnerabilities.
+The feedback loop operates based on predefined thresholds or rules, triggering actions when certain conditions are met. For instance, if the threat level exceeds a predetermined threshold, the system may automatically initiate countermeasures to neutralize the threat. This threshold-based decision-making process ensures that the system re-mains vigilant and responsive to potential security breaches, enhancing the overall security posture of the metaverse ecosystem.
+By integrating feedback loops into its security framework, the DASM Framework adopts a proactive defense strategy, capable of adapting to dynamic threat landscapes. Automated responses to security incidents minimize response times, reduce human intervention, and mitigate the impact of security breaches, ensuring the continuous protection and resilience of the metaverse ecosystem.</t>
+  </si>
+  <si>
+    <t>what is Feedback loop initiation based on paper Enhancing IoT security and healthcare data protection in the metaverse: A
+Dynamic Adaptive Security Mechanism</t>
+  </si>
+  <si>
+    <t>what is abstract from paper Enhancing IoT security through emotion recognition and
+blockchain-driven intrusion prevention</t>
+  </si>
+  <si>
+    <t>As the Internet of Things (IoT) expands, ensuring the security and privacy of interconnected devices
+poses significant challenges. Traditional intrusion detection and prevention systems (IDPS)
+for IoT rely primarily on network traffic, anomaly detection, and signature-based approaches.
+This paper addresses deficiencies in conventional infrastructure security, particularly within
+Closed-Circuit Television (CCTV) operations, to fortify IoT environments against emerging
+intrusions and ensure heightened levels of privacy and security. Traditional intrusion detection
+and prevention systems (IDPSs) for IoT primarily rely on network traffic analysis, anomaly
+detection, and signature-based approaches. However, there is a promising opportunity to
+enhance IDPS effectiveness by incorporating CCTV cameras and human-inspired techniques. We
+present a novel approach to IoT security employing CCTV cameras, Raspberry Pi, and emotion
+recognition intrusion detection and prevention. Initially, two CCTV cameras are installed and
+connected to a Raspberry Pi for video recording and preprocessing. Emotions are then detected
+using a convolutional neural network (CNN). Anomalies are classified according to predefined
+criteria based on detected emotions: individuals meeting conditions such as fear, multiple failed
+logins (greater than 2), and activity after 6 PM are classified as intruders, those meeting one
+or two criteria are labeled suspicious, while others are considered normal (non-intruders). In
+the event of suspicious activity, an alarm is automatically generated, while for intruders, an
+internet ban is also applied in addition to an alarm. Our proposed system aims to provide a
+proactive and context-aware defense mechanism against IoT intrusions by integrating machine
+learning algorithms and blockchain technology, ensuring the robustness and reliability of IoT
+security.</t>
+  </si>
+  <si>
+    <t>Raspberry Pi plays a crucial role in enhancing the capabilities of the CCTV cameras. It performs video preprocessing tasks on the
+captured video frames, improving the quality and relevance of the data for further analysis. The preprocessing pipeline for video
+frames includes the following steps:
+• Filtering: Apply spatial and temporal filters to reduce noise and enhance relevant features in the video frames. This step aids
+in the improvement of frame quality for subsequent processing.
+• Edge Detection: Detect edges and shapes in video frames using techniques such as Canny edge detection. This step is critical
+for identifying key features in the frames and supporting them in subsequent analysis.
+• Segmentation: Separate the video frames into meaningful segments or areas of interest. This step is critical for separating
+specific areas or objects for further investigation.
+• Feature Extraction: Identify and extract relevant features from the segmented regions. These elements may include facial
+landmarks, motion vectors, or other distinguishing characteristics.
+Furthermore, Raspberry Pi handles video compression tasks with algorithms such as H.264 or H.265. By reducing the size of
+the video stream without affecting quality this optimizes bandwidth usage and storage requirements. Video data is transmitted and
+stored efficiently, reducing network bandwidth utilization and storage space. Using these preprocessing techniques, the Raspberry
+Pi improves the quality and relevance of video frames captured by CCTV cameras, resulting in clean and informative data for further
+analysis in our proposed model.</t>
+  </si>
+  <si>
+    <t>explain Data preprocessing at the Raspberry Pi level based on paper Enhancing IoT security through emotion recognition and
+blockchain-driven intrusion prevention</t>
+  </si>
+  <si>
+    <t>The Internet of Things (IoT) has become deeply embedded in daily life, enabling
+pervasive collection of user and environmental data. However, securing sensor-edgecloud
+IoT architectures remains a critical challenge due to their exposure to open
+environments, resource-constrained devices, and stringent requirements for high
+throughput and real-time responsiveness. While existing software-centric security
+solutions inadequately address these constraints, we propose a hardware-enhanced
+security framework that embeds specialized security chips across all IoT layers. At the
+sensor layer, the privacy-enabled analog-to-digital converter (ADC) integrates
+lightweight encryption during data acquisition to prevent raw sensitive data exposure.
+Edge nodes employ dedicated authentication microcontroller units (MCUs) to validate
+data integrity and source legitimacy under high concurrency. Cloud servers utilize
+cryptographic system-on-chip (SoC) modules for hardware-accelerated encryption and
+fine-grained access control, enabling secure storage and dynamic policy enforcement.
+By shifting security primitives to hardware, this framework inherently mitigates
+software vulnerabilities, sustains high-throughput data processing, and minimizes
+reliance on resource-intensive software stacks, thereby establishing a robust foundation
+for next-generation IoT systems.</t>
+  </si>
+  <si>
+    <t>what is abstract from paper Hardware-enhanced Data Security for Internet of Things</t>
+  </si>
+  <si>
+    <t>Forrest et al. (2008) established the foundations of attack detec-tion through system call analysis. They used short system call trace sequences, applying both fixed-length and variable-length analysis to develop statistical intrusion-detection methods for Linux-based systems. They demonstrated that system calls are essential components for modeling how a system should function.
+Two prominent approaches are used in existing anomaly-detection systems based on system calls: (a) learning the behavior of a single process or program, and (b) considering the behavior of multiple processes, programs, or devices. In the first approach, a system call sequence from long, repeated executions of a target program or process is used. These sequences tend to be long and require segmentation into smaller patterns or activities for effective learning. For example, Subba and Gupta (2021) transformed 𝑛-grams of system call traces into fixed-length TF-IDF vectors, while Liao et al. (2022) used both fixed- and variable-length features from arbitrary-length system call sequences to train their ML model. Similarly, Carter et al. (2022) used 𝑛-grams and longest common subsequences (LCS) of system call sequences as features, along with several empirically determined parameters. In contrast, the second approach seeks to build a more generic anomaly-detection model that captures behaviors across multiple processes and devices. This involves using data sampled from various sources and extracting, deriving, or computing key features of system call sequences to build the detection model (Grimmer et al., 2018). For these ap-proaches to be practical, they must balance efficiency, lightweight implementation, high detection rates, and a low FPR.
+He et al. (2023) developed a new feature set based on the semantic grouping of system calls and used tree pruning to select important features. Similarly, Gu et al. (2021) applied natural language processing models to identify significant features of system calls.</t>
+  </si>
+  <si>
+    <t>what is Anomaly detection using system call data based on paper Integrating system calls and position-specific scoring for enhanced anomaly
+detection in Internet of Things environments</t>
+  </si>
+  <si>
+    <t>Identifying attacks on Internet of Things (IoT) systems through anomaly detection is an effective approach and
+remains a crucial area of research. The core method involves collecting system-related data during normal
+operation to establish a baseline of typical behavior and then continuously monitoring for deviations from
+this baseline. Using system call sequences for anomaly detection is a well-established and important field.
+System call sequences effectively capture the behavior of a target system at a low level, allowing identification
+of any changes in this behavior; however, these approaches face several challenges, including high falsepositive
+rates, the need for segmentation of long sequences, and the difficulty of detecting anomalies when
+the system call data comes from multiple processes. This work presents a novel anomaly-detection approach
+that uses a position-specific scoring mechanism to analyze the content and structural properties of system call
+sequences. The proposed approach addresses key challenges in this field, including fixed-length segmentation of
+system call sequences, predetermined anomaly-detection thresholds, the detection of anomalies in both single
+and multiple processes, and high false-positive rates. We extensively evaluated the proposed approach using
+system-call-specific public datasets (ADFA-LD and UNM) of a diverse nature. The performance of the proposed
+content-based, structure-based, and combined content- and structure-based anomaly-detection methods was
+evaluated using ten-fold cross-validation. The proposed anomaly-detection approach achieves an impressive
+detection rate of 1.0, along with exceptionally low false-positive rates of 0.001 and 0.017 when evaluated on
+the UNM and ADFA-LD datasets, respectively.</t>
+  </si>
+  <si>
+    <t>what is abstract from paper Integrating system calls and position-specific scoring for enhanced anomaly
+detection in Internet of Things environments</t>
+  </si>
+  <si>
+    <t>Position-based scoring techniques were initially developed to assess the similarity of protein sequences (Zhu et al., 2019). These tech-niques have since proven valuable in a range of protein-analysis tasks, including secondary-structure prediction (Jones, 1999), binding-site identification (Chen and Jeong, 2009), and fold recognition (Sharma et al., 2013). The fundamental requirement for this approach is that all sequences must be of equal length, and that similar symbols across sequences must occupy the same positions. The method constructs a matrix of aligned, fixed-length sequences and calculates the probability of each symbol appearing at each position. These probabilities form a PSS, which is then used to evaluate the similarity of new sequences. The overall score for a sequence is obtained by combining the PSS values of its constituent symbols. A higher score indicates that the sequence closely resembles those used to construct the matrix, particularly when the symbol positions align well; otherwise, the score remains low.</t>
+  </si>
+  <si>
+    <t>what is Position-specific scoring based on paper Integrating system calls and position-specific scoring for enhanced anomaly
+detection in Internet of Things environments</t>
+  </si>
+  <si>
+    <t>The IoT is an advanced digital domain that connects devices and
+physical objects to the digital realm (Internet). The fluid data sharing
+that this interconnection enables has an impact on the different IoT
+areas, such as healthcare, transportation, smart cities, smart homes,
+vehicles, agriculture, nursing, manufacturing, etc. However, there are
+significant concerns about the security and privacy of the collected
+and shared data because of the rapid expansion of IoT. Robust IoT
+data management becomes important in Fog and Cloud computing
+environments. Large volumes of data are being generated through the
+growing number of devices, thus, it is critical to control this data
+efficiently and securely while facilitating access to pertinent data. Fog
+computing facilitates computation and enables real-time processing
+regarding data sources, whereas cloud computing offers a reliable
+and centralized solution for storing and analyzing IoT-generated data.
+Both approaches take into account different aspects like scalability and
+security while addressing data storage, analysis, and access challenges.
+In this research study, we will analyze the optimization of security
+component placement in an IoT environment, taking into account
+many security placement technologies to improve security in cloud computing systems, as well as optimization techniques to guarantee the
+greatest availability. However, it is a top concern to implement robust
+data confidentiality mechanisms within the IoT. Private and sensitive
+information extracted from connected devices needs strong protection
+to avoid unauthorized access and unwanted use. In addition, access
+control AC builds complex issues in a dynamic and distributed IoT environment.
+A security problem in a device can propagate throughout the
+network, causing a large amount of damage. There are multiple access
+control-based research mechanisms for data protection. Therefore, it is
+important to include new research on different technologies to improve
+privacy in cloud computing [1]. A set of rules and procedures in access
+control can provide unauthorized users access to different data that
+gives data confidentiality, integrity, and security</t>
+  </si>
+  <si>
+    <t>what is Context and issue based on paper New privacy-respecting access control-based approach for data placement in
+an Internet of Things environment</t>
+  </si>
+  <si>
+    <t>access control-based approach for secure data placement in IoT envi-ronments. By integrating Formal Concept Analysis (FCA) with Role-Based Access Control (RBAC), our method enhances data confiden-tiality while optimizing access control mechanisms. The experimental results demonstrate that DPPAC outperforms traditional RBAC and FCA techniques in key metrics such as Authorization Rate (AR), Rejection Rate (RR), Precision, Recall, and F-measure, proving its effectiveness in minimizing unauthorized access risks.
+Our DPPAC approach is designed to complement, not replace, other existing protective mechanisms. While it significantly improves access control and data confidentiality, it does not address all security risks and therefore requires the integration of additional security mecha-nisms such as trust management and real-time monitoring to provide a comprehensive protection framework for IoT environments. Its goal is to improve access control by reducing role misassignments and en-hancing data confidentiality, ensuring robust security for sensitive data in IoT ecosystems while maintaining efficient and authorized access.
+The findings highlight the potential of combining mathematical modeling (FCA) with access control policies (RBAC) to address evolving security challenges in IoT.
+Future work could explore scalability in larger IoT networks and adaptation to dynamic access control scenarios, further strengthening data privacy in next-generation internet environments.
+Ultimately, DPPAC provides a reliable, efficient, and privacy-aware solution for securing sensitive data in IoT, paving the way for safer and more trustworthy smart ecosystems.</t>
+  </si>
+  <si>
+    <t>what is Summary from Conclusion and future work based on paper New privacy-respecting access control-based approach for data placement in
+an Internet of Things environment</t>
+  </si>
+  <si>
+    <t>As the main contribution, in this work, we have proposed a new Privacy-Respecting Access Control-based Approach for Data Placement in an IoT Environment.
+The first originality in our research is the combination of Formal Concept Analysis (FCA) and Role-Based Access Control (RBAC) to im-plement an effective data confidentiality and access control mechanism. Despite traditional approaches, our approach organizes and prioritizes relationships between objects and their attributes (fog and cloud nodes, respectively, in our work) in a multi-cloud context, enabling effective role and permissions assignment.
+The second originality is that our approach provides scalability by ensuring the flexible inclusion of additional elements (objects, roles, permissions) as the IoT environment evolves. This adaptability makes it suitable for solving complex and new requirements.
+The main contributions of our work, to address the above chal-lenges, are as follows:
+•
+To propose a new DPPAC model to improve data confidentiality by structuring access controls based on hierarchical relationships between IoT entities (respectively fog and cloud nodes).
+•
+To provide a flexible and adaptable framework that supports the emerging IoT environments by efficient and robust access control systems.
+•
+To implement and evaluate our proposed approach to demon-strate its effectiveness based on key indicators such as access control and data confidentiality.</t>
+  </si>
+  <si>
+    <t>what is Contributions from paper New privacy-respecting access control-based approach for data placement in
+an Internet of Things environment</t>
+  </si>
+  <si>
+    <t>The future internet landscape is increasingly dependent on social networks and the Internet of Things (IoT),
+leveraging diverse communication technologies. While early internet usage primarily involved web browsing,
+multimedia services, and social networking, the rapid proliferation of the IoT has made data confidentiality
+and security paramount.
+This paper presents a novel approach that integrates Formal Concept Analysis (FCA) with Role-Based
+Access Control (RBAC) to strengthen access control and optimize data confidentiality in IoT environments.
+Our proposed Data Placement in IoT using Privacy-respecting Access Control (DPPAC) framework addresses
+two critical challenges: minimizing unauthorized access risks and ensuring robust data confidentiality through
+optimal security component placement.
+A comprehensive evaluation demonstrates DPPAC’s superiority over traditional RBAC and FCA methods
+across key metrics, including Authorization Rate (AR), Rejection Rate (RR), Precision, Recall, and 𝐹measure.
+Experimental results show that DPPAC achieves significantly higher AR and lower RR compared to traditional
+approaches, confirming its enhanced security capabilities.</t>
+  </si>
+  <si>
+    <t>what is the abstract from paper New privacy-respecting access control-based approach for data placement in
+an Internet of Things environment</t>
+  </si>
+  <si>
+    <t>Before implementing our solution, we will prepare our proper dataset based on the Kaggle Cloud-Fog Computing Dataset https://www.kaggle.com/datasets/sachin26240/vehicularfogcomputing. This database is designed to store and manage information related to access permissions and roles in a fog node-based access control system. Our generated dataset consists of a variable number of FN and CN to determine their effects on the privacy and confidentiality of sensitive data accessed between nodes within an IoT environment. We vary the number of FN and at the same time the number of CN randomly, as indicated in Table 3.
+The values of each fog and cloud node are chosen randomly from the range [500, 5000]. To improve the security and confidentiality of sensitive data at the access control of these nodes and determine the optimal number of them required for the IoT environment, ensuring geographic proximity to reduce latency, implementing robust security measures to protect sensitive data, and ensuring sufficient redundancy, as follows:
+•
+Geographic proximity: By ensuring that the FN and CN are de-ployed close to IoT devices, the risks of latency and network dis-ruption are reduced, which can contribute to enhancing security by minimizing delays in transmitting sensitive data.
+•
+Security: Ensuring that CN has robust security measures to pro-tect stored data, such as monitoring of unauthorized access, en-sures the confidentiality of sensitive information, and reduces the risks of data breaches.
+•
+Redundancy: Ensures continuous availability of the system in case of failure or incident. By having redundant nodes, the re-liability of the system is strengthened, and the risks of disruption to sensitive data are reduced.
+Our IoT data placement optimization solution employs FCA-based access control (RBAC), which follows a systematic approach to collect relevant access permission data. Initially, we identify network fog and cloud nodes, roles, and their corresponding permissions. Then, roles are randomly assigned to Cloud nodes, each with specific permissions. These permissions are defined based on preset criteria such as read-only, create, delete, etc. Subsequently, we create a binary access matrix to illustrate permissions between Fog and Cloud nodes, facilitating a clear understanding of access dynamics in the IoT network. Overall, our data collection method forms a robust basis for analyzing the effectiveness and security of our AC approach.</t>
+  </si>
+  <si>
+    <t>what Data collection who use on paper New privacy-respecting access control-based approach for data placement in
+an Internet of Things environment</t>
+  </si>
 </sst>
 </file>
 
@@ -926,11 +2096,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -946,10 +2120,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1269,7 +2439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3744A4C2-A66F-440C-B54D-D3DC708D0F68}">
-  <dimension ref="A2:F33"/>
+  <dimension ref="A2:F102"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
@@ -1542,6 +2712,558 @@
       </c>
       <c r="C33" s="1" t="s">
         <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="302.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="374.4" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="388.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="360" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="331.2" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="302.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="360" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="331.2" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A57" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="302.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A59" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="302.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="360" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" s="3" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A68" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="360" x14ac:dyDescent="0.3">
+      <c r="A71" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="331.2" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="288" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="244.8" x14ac:dyDescent="0.3">
+      <c r="A75" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A76" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A77" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="288" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="A79" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A80" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="374.4" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A82" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="A83" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" ht="374.4" x14ac:dyDescent="0.3">
+      <c r="A84" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A85" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A86" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A87" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" ht="216" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="A89" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" ht="273.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A90" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A91" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A94" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A96" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" ht="273.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A99" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A100" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" ht="331.2" x14ac:dyDescent="0.3">
+      <c r="A101" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A102" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -1583,11 +3305,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5146d105-7d5f-496c-bd31-80ca7e72687a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1830,27 +3553,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5146d105-7d5f-496c-bd31-80ca7e72687a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93A08990-164D-4746-AA33-F52EDACD1948}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACE9AC90-BA89-410A-B600-14200351DC12}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="5146d105-7d5f-496c-bd31-80ca7e72687a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3de855c3-8ecd-4254-b07d-50bb50556e99"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1875,9 +3588,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACE9AC90-BA89-410A-B600-14200351DC12}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93A08990-164D-4746-AA33-F52EDACD1948}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="3de855c3-8ecd-4254-b07d-50bb50556e99"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="5146d105-7d5f-496c-bd31-80ca7e72687a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>